<commit_message>
BAADTbVT, BCDTRTSY, BHNVFEAL, BNVFE, SYFAFE calibrate aircraft
</commit_message>
<xml_diff>
--- a/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
+++ b/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\trans\BHNVFEAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29D056D9-250C-41EE-99AC-A85FBBA54DAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A986EBF-6A38-4458-9EF9-9AB3274F4F22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="5" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1290,7 +1290,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1327,17 +1327,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="154" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="155" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="11" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="11" fontId="41" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="41" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="30" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="43" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="154" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="156">
     <cellStyle name="20% - Accent1 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -9012,6 +9008,7 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="2" max="2" width="21.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:34" ht="30">
@@ -9430,7 +9427,7 @@
       <c r="A5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="32">
         <f>Extrapolations!Q6</f>
         <v>4.3905417607014065E-4</v>
       </c>
@@ -17158,104 +17155,104 @@
       <c r="AJ15" s="4"/>
       <c r="AK15" s="4"/>
     </row>
-    <row r="16" spans="1:37" s="36" customFormat="1">
-      <c r="A16" s="36" t="s">
+    <row r="16" spans="1:37" s="31" customFormat="1">
+      <c r="A16" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="31" t="s">
         <v>22</v>
       </c>
-      <c r="C16" s="36" t="s">
+      <c r="C16" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="D16" s="36">
+      <c r="D16" s="31">
         <v>3.5120030000000001E-3</v>
       </c>
-      <c r="E16" s="36">
+      <c r="E16" s="31">
         <v>3.3663400000000002E-3</v>
       </c>
-      <c r="F16" s="36">
+      <c r="F16" s="31">
         <v>3.3698929999999997E-3</v>
       </c>
-      <c r="G16" s="36">
+      <c r="G16" s="31">
         <v>3.3734500000000001E-3</v>
       </c>
-      <c r="H16" s="36">
+      <c r="H16" s="31">
         <v>3.3770099999999997E-3</v>
       </c>
-      <c r="I16" s="36">
+      <c r="I16" s="31">
         <v>3.3805740000000003E-3</v>
       </c>
-      <c r="J16" s="36">
+      <c r="J16" s="31">
         <v>3.3841420000000001E-3</v>
       </c>
-      <c r="K16" s="36">
+      <c r="K16" s="31">
         <v>3.3877130000000001E-3</v>
       </c>
-      <c r="L16" s="36">
+      <c r="L16" s="31">
         <v>3.391289E-3</v>
       </c>
-      <c r="M16" s="36">
+      <c r="M16" s="31">
         <v>3.3948680000000001E-3</v>
       </c>
-      <c r="N16" s="36">
+      <c r="N16" s="31">
         <v>3.3984510000000002E-3</v>
       </c>
-      <c r="O16" s="36">
+      <c r="O16" s="31">
         <v>3.4020370000000001E-3</v>
       </c>
-      <c r="P16" s="36">
+      <c r="P16" s="31">
         <v>3.405628E-3</v>
       </c>
-      <c r="Q16" s="36">
+      <c r="Q16" s="31">
         <v>3.4092220000000004E-3</v>
       </c>
-      <c r="R16" s="36">
+      <c r="R16" s="31">
         <v>3.41282E-3</v>
       </c>
-      <c r="S16" s="36">
+      <c r="S16" s="31">
         <v>3.4164219999999997E-3</v>
       </c>
-      <c r="T16" s="36">
+      <c r="T16" s="31">
         <v>3.420027E-3</v>
       </c>
-      <c r="U16" s="36">
+      <c r="U16" s="31">
         <v>3.4236369999999998E-3</v>
       </c>
-      <c r="V16" s="36">
+      <c r="V16" s="31">
         <v>3.4272499999999997E-3</v>
       </c>
-      <c r="W16" s="36">
+      <c r="W16" s="31">
         <v>3.4308670000000002E-3</v>
       </c>
-      <c r="X16" s="36">
+      <c r="X16" s="31">
         <v>3.4344879999999999E-3</v>
       </c>
-      <c r="Y16" s="36">
+      <c r="Y16" s="31">
         <v>3.438113E-3</v>
       </c>
-      <c r="Z16" s="36">
+      <c r="Z16" s="31">
         <v>3.4417409999999999E-3</v>
       </c>
-      <c r="AA16" s="36">
+      <c r="AA16" s="31">
         <v>3.4453729999999998E-3</v>
       </c>
-      <c r="AB16" s="36">
+      <c r="AB16" s="31">
         <v>3.4490099999999997E-3</v>
       </c>
-      <c r="AC16" s="36">
+      <c r="AC16" s="31">
         <v>3.4526489999999999E-3</v>
       </c>
-      <c r="AD16" s="36">
+      <c r="AD16" s="31">
         <v>3.456293E-3</v>
       </c>
-      <c r="AE16" s="36">
+      <c r="AE16" s="31">
         <v>3.4599410000000002E-3</v>
       </c>
-      <c r="AF16" s="36">
+      <c r="AF16" s="31">
         <v>3.4635930000000001E-3</v>
       </c>
-      <c r="AG16" s="36">
+      <c r="AG16" s="31">
         <v>3.467248E-3</v>
       </c>
     </row>
@@ -18533,16 +18530,16 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>1.2987877392438942E-3</v>
+        <v>1.3768785799698285E-3</v>
       </c>
       <c r="C4">
-        <v>4.0416928234185732E-4</v>
+        <v>4.2847034255362628E-4</v>
       </c>
       <c r="D4">
-        <v>4.0416928234185732E-4</v>
+        <v>4.2847034255362628E-4</v>
       </c>
       <c r="E4">
-        <v>4.0416928234185732E-4</v>
+        <v>4.2847034255362628E-4</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -18551,7 +18548,7 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>1.2125078470255717E-3</v>
+        <v>1.2854110276608786E-3</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -18715,16 +18712,16 @@
         <v>7</v>
       </c>
       <c r="B12">
-        <v>4.6228905610524535E-4</v>
+        <v>5.4991909569712227E-4</v>
       </c>
       <c r="C12">
-        <v>1.4385956257126716E-4</v>
+        <v>1.7112912259502911E-4</v>
       </c>
       <c r="D12">
-        <v>1.4385956257126716E-4</v>
+        <v>1.7112912259502911E-4</v>
       </c>
       <c r="E12">
-        <v>1.4385956257126716E-4</v>
+        <v>1.7112912259502911E-4</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -18733,7 +18730,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>4.3157868771380144E-4</v>
+        <v>5.1338736778508724E-4</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -19208,9 +19205,6 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="15" max="15" width="11.42578125" customWidth="1"/>
-    <col min="28" max="39" width="9.140625" style="31"/>
-    <col min="40" max="40" width="8.7109375" style="31"/>
-    <col min="42" max="42" width="9.140625" style="31"/>
     <col min="43" max="43" width="9.140625" style="23"/>
   </cols>
   <sheetData>
@@ -19290,49 +19284,49 @@
       <c r="AA1">
         <v>2007</v>
       </c>
-      <c r="AB1" s="31">
+      <c r="AB1">
         <v>2008</v>
       </c>
-      <c r="AC1" s="31">
+      <c r="AC1">
         <v>2009</v>
       </c>
-      <c r="AD1" s="31">
+      <c r="AD1">
         <v>2010</v>
       </c>
-      <c r="AE1" s="31">
+      <c r="AE1">
         <v>2011</v>
       </c>
-      <c r="AF1" s="31">
+      <c r="AF1">
         <v>2012</v>
       </c>
-      <c r="AG1" s="31">
+      <c r="AG1">
         <v>2013</v>
       </c>
-      <c r="AH1" s="31">
+      <c r="AH1">
         <v>2014</v>
       </c>
-      <c r="AI1" s="31">
+      <c r="AI1">
         <v>2015</v>
       </c>
-      <c r="AJ1" s="31">
+      <c r="AJ1">
         <v>2016</v>
       </c>
-      <c r="AK1" s="31">
+      <c r="AK1">
         <v>2017</v>
       </c>
-      <c r="AL1" s="31">
+      <c r="AL1">
         <v>2018</v>
       </c>
-      <c r="AM1" s="31">
+      <c r="AM1">
         <v>2019</v>
       </c>
-      <c r="AN1" s="31">
+      <c r="AN1">
         <v>2020</v>
       </c>
       <c r="AO1">
         <v>2021</v>
       </c>
-      <c r="AP1" s="31">
+      <c r="AP1">
         <v>2022</v>
       </c>
       <c r="AQ1" s="23">
@@ -19455,55 +19449,55 @@
         <f>Calculations!C16</f>
         <v>3.142498616321923E-4</v>
       </c>
-      <c r="AB2" s="32">
+      <c r="AB2" s="26">
         <f t="shared" ref="AB2:AO2" si="0">($AR$2-$AA$2)/COUNT($AB$1:$AR$1)+AA2</f>
         <v>3.1779260113808729E-4</v>
       </c>
-      <c r="AC2" s="32">
+      <c r="AC2" s="26">
         <f t="shared" si="0"/>
         <v>3.2133534064398227E-4</v>
       </c>
-      <c r="AD2" s="32">
+      <c r="AD2" s="26">
         <f t="shared" si="0"/>
         <v>3.2487808014987726E-4</v>
       </c>
-      <c r="AE2" s="32">
+      <c r="AE2" s="26">
         <f t="shared" si="0"/>
         <v>3.2842081965577224E-4</v>
       </c>
-      <c r="AF2" s="32">
+      <c r="AF2" s="26">
         <f t="shared" si="0"/>
         <v>3.3196355916166722E-4</v>
       </c>
-      <c r="AG2" s="32">
+      <c r="AG2" s="26">
         <f t="shared" si="0"/>
         <v>3.3550629866756221E-4</v>
       </c>
-      <c r="AH2" s="32">
+      <c r="AH2" s="26">
         <f t="shared" si="0"/>
         <v>3.3904903817345719E-4</v>
       </c>
-      <c r="AI2" s="32">
+      <c r="AI2" s="26">
         <f t="shared" si="0"/>
         <v>3.4259177767935218E-4</v>
       </c>
-      <c r="AJ2" s="32">
+      <c r="AJ2" s="26">
         <f t="shared" si="0"/>
         <v>3.4613451718524716E-4</v>
       </c>
-      <c r="AK2" s="32">
+      <c r="AK2" s="26">
         <f t="shared" si="0"/>
         <v>3.4967725669114214E-4</v>
       </c>
-      <c r="AL2" s="32">
+      <c r="AL2" s="26">
         <f t="shared" si="0"/>
         <v>3.5321999619703713E-4</v>
       </c>
-      <c r="AM2" s="32">
+      <c r="AM2" s="26">
         <f t="shared" si="0"/>
         <v>3.5676273570293211E-4</v>
       </c>
-      <c r="AN2" s="32">
+      <c r="AN2" s="26">
         <f t="shared" si="0"/>
         <v>3.603054752088271E-4</v>
       </c>
@@ -19511,11 +19505,11 @@
         <f t="shared" si="0"/>
         <v>3.6384821471472208E-4</v>
       </c>
-      <c r="AP2" s="32">
+      <c r="AP2" s="26">
         <f>($AR$2-$AA$2)/COUNT($AB$1:$AR$1)+AO2</f>
         <v>3.6739095422061706E-4</v>
       </c>
-      <c r="AQ2" s="32">
+      <c r="AQ2" s="26">
         <f>($AR$2-$AA$2)/COUNT($AB$1:$AR$1)+AP2</f>
         <v>3.7093369372651205E-4</v>
       </c>
@@ -19661,71 +19655,71 @@
       <c r="X3" s="9"/>
       <c r="Y3" s="9"/>
       <c r="Z3" s="9"/>
-      <c r="AA3" s="30" cm="1">
+      <c r="AA3" s="4" cm="1">
         <f t="array" ref="AA3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AA1)</f>
         <v>6.2736507518388511E-5</v>
       </c>
-      <c r="AB3" s="30" cm="1">
+      <c r="AB3" s="4" cm="1">
         <f t="array" ref="AB3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AB1)</f>
         <v>6.3701994710036553E-5</v>
       </c>
-      <c r="AC3" s="30" cm="1">
+      <c r="AC3" s="4" cm="1">
         <f t="array" ref="AC3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AC1)</f>
         <v>6.4667481901684379E-5</v>
       </c>
-      <c r="AD3" s="30" cm="1">
+      <c r="AD3" s="4" cm="1">
         <f t="array" ref="AD3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AD1)</f>
         <v>6.5632969093332421E-5</v>
       </c>
-      <c r="AE3" s="30" cm="1">
+      <c r="AE3" s="4" cm="1">
         <f t="array" ref="AE3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AE1)</f>
         <v>6.6598456284980246E-5</v>
       </c>
-      <c r="AF3" s="30" cm="1">
+      <c r="AF3" s="4" cm="1">
         <f t="array" ref="AF3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AF1)</f>
         <v>6.7563943476628288E-5</v>
       </c>
-      <c r="AG3" s="30" cm="1">
+      <c r="AG3" s="4" cm="1">
         <f t="array" ref="AG3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AG1)</f>
         <v>6.8529430668276114E-5</v>
       </c>
-      <c r="AH3" s="30" cm="1">
+      <c r="AH3" s="4" cm="1">
         <f t="array" ref="AH3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AH1)</f>
         <v>6.9494917859924156E-5</v>
       </c>
-      <c r="AI3" s="30" cm="1">
+      <c r="AI3" s="4" cm="1">
         <f t="array" ref="AI3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AI1)</f>
         <v>7.0460405051572198E-5</v>
       </c>
-      <c r="AJ3" s="30" cm="1">
+      <c r="AJ3" s="4" cm="1">
         <f t="array" ref="AJ3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AJ1)</f>
         <v>7.1425892243220023E-5</v>
       </c>
-      <c r="AK3" s="30" cm="1">
+      <c r="AK3" s="4" cm="1">
         <f t="array" ref="AK3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AK1)</f>
         <v>7.2391379434868066E-5</v>
       </c>
-      <c r="AL3" s="30" cm="1">
+      <c r="AL3" s="4" cm="1">
         <f t="array" ref="AL3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AL1)</f>
         <v>7.3356866626515891E-5</v>
       </c>
-      <c r="AM3" s="30" cm="1">
+      <c r="AM3" s="4" cm="1">
         <f t="array" ref="AM3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AM1)</f>
         <v>7.4322353818163933E-5</v>
       </c>
-      <c r="AN3" s="30" cm="1">
+      <c r="AN3" s="4" cm="1">
         <f t="array" ref="AN3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AN1)</f>
         <v>7.5287841009811758E-5</v>
       </c>
-      <c r="AO3" s="30" cm="1">
+      <c r="AO3" s="4" cm="1">
         <f t="array" ref="AO3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AO1)</f>
         <v>7.6253328201459801E-5</v>
       </c>
-      <c r="AP3" s="30" cm="1">
+      <c r="AP3" s="4" cm="1">
         <f t="array" ref="AP3">TREND($AR$3:$AV$3,$AR$1:$AV$1,AP1)</f>
         <v>7.6915445435660028E-5</v>
       </c>
-      <c r="AQ3" s="30" cm="1">
+      <c r="AQ3" s="4" cm="1">
         <f t="array" ref="AQ3">TREND($AR$3:$AV$3,$AR$1:$AV$1,AQ1)</f>
         <v>7.8010948323356793E-5</v>
       </c>
@@ -19920,67 +19914,67 @@
         <f t="shared" si="1"/>
         <v>9.9033214307749757E-4</v>
       </c>
-      <c r="AB4" s="30">
+      <c r="AB4" s="4">
         <f t="shared" si="1"/>
         <v>9.9152077795891806E-4</v>
       </c>
-      <c r="AC4" s="30">
+      <c r="AC4" s="4">
         <f t="shared" si="1"/>
         <v>9.9270941284033856E-4</v>
       </c>
-      <c r="AD4" s="30">
+      <c r="AD4" s="4">
         <f t="shared" si="1"/>
         <v>9.9389804772175906E-4</v>
       </c>
-      <c r="AE4" s="30">
+      <c r="AE4" s="4">
         <f t="shared" si="1"/>
         <v>9.9508668260317955E-4</v>
       </c>
-      <c r="AF4" s="30">
+      <c r="AF4" s="4">
         <f t="shared" si="1"/>
         <v>9.9627531748460005E-4</v>
       </c>
-      <c r="AG4" s="30">
+      <c r="AG4" s="4">
         <f>AG5/AH5*AH4</f>
         <v>9.9746395236602055E-4</v>
       </c>
-      <c r="AH4" s="30">
+      <c r="AH4" s="4">
         <f t="shared" si="1"/>
         <v>9.9865258724744104E-4</v>
       </c>
-      <c r="AI4" s="30">
+      <c r="AI4" s="4">
         <f t="shared" si="1"/>
         <v>9.9984122212886154E-4</v>
       </c>
-      <c r="AJ4" s="30">
+      <c r="AJ4" s="4">
         <f>AJ5/AK5*AK4</f>
         <v>1.001029857010282E-3</v>
       </c>
-      <c r="AK4" s="33">
+      <c r="AK4" s="19">
         <f>AK5/AL5*AL4</f>
         <v>1.0022184918917025E-3</v>
       </c>
-      <c r="AL4" s="33">
+      <c r="AL4" s="19">
         <f>AL5/AM5*AM4</f>
         <v>1.003407126773123E-3</v>
       </c>
-      <c r="AM4" s="33">
+      <c r="AM4" s="19">
         <f>AM5/AN5*AN4</f>
         <v>1.0045957616545435E-3</v>
       </c>
-      <c r="AN4" s="33">
+      <c r="AN4" s="19">
         <f t="shared" ref="AN4:AQ4" si="2">AN5/AO5*AO4</f>
         <v>1.005784396535964E-3</v>
       </c>
-      <c r="AO4" s="33">
+      <c r="AO4" s="19">
         <f t="shared" si="2"/>
         <v>1.0069730314173845E-3</v>
       </c>
-      <c r="AP4" s="33">
+      <c r="AP4" s="19">
         <f t="shared" si="2"/>
         <v>1.008161666298805E-3</v>
       </c>
-      <c r="AQ4" s="33">
+      <c r="AQ4" s="19">
         <f t="shared" si="2"/>
         <v>1.0105389360616456E-3</v>
       </c>
@@ -20160,7 +20154,7 @@
         <v>7.8134709903309753E-4</v>
       </c>
       <c r="X5" s="4">
-        <f t="shared" ref="X5:AP5" si="4">($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+W5</f>
+        <f t="shared" ref="X5:AN5" si="4">($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+W5</f>
         <v>7.8228942606352163E-4</v>
       </c>
       <c r="Y5" s="4">
@@ -20231,7 +20225,7 @@
         <f>($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+AN5</f>
         <v>7.9830898558073125E-4</v>
       </c>
-      <c r="AP5" s="30">
+      <c r="AP5" s="4">
         <f>($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+AO5</f>
         <v>7.9925131261115534E-4</v>
       </c>
@@ -20370,111 +20364,111 @@
       <c r="M6" s="9"/>
       <c r="N6" s="9"/>
       <c r="O6" s="9"/>
-      <c r="P6" s="30">
+      <c r="P6" s="4">
         <f t="shared" ref="P6:AM6" si="5">TREND($AQ6:$BR6,$AQ$1:$BR$1,P$1)</f>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="Q6" s="30">
+      <c r="Q6" s="4">
+        <f>TREND($AQ6:$BR6,$AQ$1:$BR$1,Q$1)</f>
+        <v>4.3905417607014065E-4</v>
+      </c>
+      <c r="R6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="R6" s="30">
+      <c r="S6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="S6" s="30">
+      <c r="T6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="T6" s="30">
+      <c r="U6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="U6" s="30">
+      <c r="V6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="V6" s="30">
+      <c r="W6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="W6" s="30">
+      <c r="X6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="X6" s="30">
+      <c r="Y6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="Y6" s="30">
+      <c r="Z6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="Z6" s="30">
+      <c r="AA6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AA6" s="30">
+      <c r="AB6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AB6" s="30">
+      <c r="AC6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AC6" s="30">
+      <c r="AD6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AD6" s="30">
+      <c r="AE6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AE6" s="30">
+      <c r="AF6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AF6" s="30">
+      <c r="AG6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AG6" s="30">
+      <c r="AH6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AH6" s="30">
+      <c r="AI6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AI6" s="30">
+      <c r="AJ6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AJ6" s="30">
+      <c r="AK6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AK6" s="30">
+      <c r="AL6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AL6" s="30">
+      <c r="AM6" s="4">
         <f t="shared" si="5"/>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AM6" s="30">
-        <f t="shared" si="5"/>
-        <v>4.3905417607014065E-4</v>
-      </c>
-      <c r="AN6" s="30">
+      <c r="AN6" s="4">
         <f>TREND($AQ6:$BR6,$AQ$1:$BR$1,AN$1)</f>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AO6" s="30">
+      <c r="AO6" s="4">
         <f t="shared" ref="AO6:AP6" si="6">TREND($AQ6:$BR6,$AQ$1:$BR$1,AO$1)</f>
         <v>4.3905417607014065E-4</v>
       </c>
-      <c r="AP6" s="30">
+      <c r="AP6" s="4">
         <f t="shared" si="6"/>
         <v>4.3905417607014065E-4</v>
       </c>
@@ -20934,55 +20928,55 @@
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AB8" s="30">
+      <c r="AB8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AC8" s="30">
+      <c r="AC8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AD8" s="30">
+      <c r="AD8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AE8" s="30">
+      <c r="AE8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AF8" s="30">
+      <c r="AF8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AG8" s="30">
+      <c r="AG8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AH8" s="30">
+      <c r="AH8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AI8" s="30">
+      <c r="AI8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AJ8" s="30">
+      <c r="AJ8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AK8" s="30">
+      <c r="AK8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AL8" s="30">
+      <c r="AL8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AM8" s="30">
+      <c r="AM8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AN8" s="30">
+      <c r="AN8" s="4">
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
@@ -20990,7 +20984,7 @@
         <f t="shared" si="8"/>
         <v>7.1745362435245036E-5</v>
       </c>
-      <c r="AP8" s="30">
+      <c r="AP8" s="4">
         <f>AO8</f>
         <v>7.1745362435245036E-5</v>
       </c>
@@ -21207,55 +21201,55 @@
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AB9" s="30">
+      <c r="AB9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AC9" s="30">
+      <c r="AC9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AD9" s="30">
+      <c r="AD9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AE9" s="30">
+      <c r="AE9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AF9" s="30">
+      <c r="AF9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AG9" s="30">
+      <c r="AG9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AH9" s="30">
+      <c r="AH9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AI9" s="30">
+      <c r="AI9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AJ9" s="30">
+      <c r="AJ9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AK9" s="30">
+      <c r="AK9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AL9" s="30">
+      <c r="AL9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AM9" s="30">
+      <c r="AM9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AN9" s="30">
+      <c r="AN9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
@@ -21263,7 +21257,7 @@
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
-      <c r="AP9" s="30">
+      <c r="AP9" s="4">
         <f t="shared" si="9"/>
         <v>7.5686214263268839E-4</v>
       </c>
@@ -21936,151 +21930,151 @@
       <c r="D12" s="9"/>
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
-      <c r="G12" s="30">
-        <f t="shared" ref="G12:AN12" si="11">TREND($AR12:$BR12,$AR$1:$BR$1,G$1)</f>
+      <c r="G12" s="4">
+        <f t="shared" ref="G12" si="11">TREND($AR12:$BR12,$AR$1:$BR$1,G$1)</f>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="H12" s="30">
+      <c r="H12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="I12" s="30">
+      <c r="I12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="J12" s="30">
+      <c r="J12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="K12" s="30">
+      <c r="K12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="L12" s="30">
+      <c r="L12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="M12" s="30">
+      <c r="M12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="N12" s="30">
+      <c r="N12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="O12" s="30">
+      <c r="O12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="P12" s="30">
+      <c r="P12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="Q12" s="30">
+      <c r="Q12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="R12" s="30">
+      <c r="R12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="S12" s="30">
+      <c r="S12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="T12" s="30">
+      <c r="T12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="U12" s="30">
+      <c r="U12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="V12" s="30">
+      <c r="V12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="W12" s="30">
+      <c r="W12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="X12" s="30">
+      <c r="X12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="Y12" s="30">
+      <c r="Y12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="Z12" s="30">
+      <c r="Z12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AA12" s="30">
+      <c r="AA12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AB12" s="30">
+      <c r="AB12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AC12" s="30">
+      <c r="AC12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AD12" s="30">
+      <c r="AD12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AE12" s="30">
+      <c r="AE12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AF12" s="30">
+      <c r="AF12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AG12" s="30">
+      <c r="AG12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AH12" s="30">
+      <c r="AH12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AI12" s="30">
+      <c r="AI12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AJ12" s="30">
+      <c r="AJ12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AK12" s="30">
+      <c r="AK12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AL12" s="30">
+      <c r="AL12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AM12" s="30">
+      <c r="AM12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AN12" s="30">
+      <c r="AN12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AO12" s="30">
+      <c r="AO12" s="4">
         <f>TREND($AR12:$BR12,$AR$1:$BR$1,AO$1)</f>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AP12" s="30">
+      <c r="AP12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
-      <c r="AQ12" s="30">
+      <c r="AQ12" s="4">
         <f t="shared" si="10"/>
         <v>5.2112239143541636E-3</v>
       </c>
@@ -22464,55 +22458,55 @@
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AB14" s="31">
+      <c r="AB14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AC14" s="31">
+      <c r="AC14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AD14" s="31">
+      <c r="AD14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AE14" s="31">
+      <c r="AE14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AF14" s="31">
+      <c r="AF14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AG14" s="31">
+      <c r="AG14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AH14" s="31">
+      <c r="AH14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AI14" s="31">
+      <c r="AI14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AJ14" s="31">
+      <c r="AJ14">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AK14" s="34">
+      <c r="AK14" s="30">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AL14" s="34">
+      <c r="AL14" s="30">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AM14" s="34">
+      <c r="AM14" s="30">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="AN14" s="34">
+      <c r="AN14" s="30">
         <f>$AO14</f>
         <v>0</v>
       </c>
@@ -22520,7 +22514,7 @@
         <f>BNVFE!D20</f>
         <v>0</v>
       </c>
-      <c r="AP14" s="35">
+      <c r="AP14" s="11">
         <f>BNVFE!E20</f>
         <v>0</v>
       </c>
@@ -22641,7 +22635,7 @@
     <row r="15" spans="1:72">
       <c r="E15" s="21"/>
       <c r="X15" s="4"/>
-      <c r="AH15" s="30"/>
+      <c r="AH15" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
BAADTbVT, SYFAFE for ships calibration
</commit_message>
<xml_diff>
--- a/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
+++ b/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\trans\BHNVFEAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51991E45-905E-42B8-9F2E-7BCF8D3BD7AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28AC5378-ED77-42E3-8839-619BE7FF2F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -18763,16 +18763,16 @@
         <v>17</v>
       </c>
       <c r="B14">
-        <v>1.5549894526873581E-2</v>
+        <v>1.5610349625283874E-2</v>
       </c>
       <c r="C14">
-        <v>4.8389660000000001E-3</v>
+        <v>4.8577789999999996E-3</v>
       </c>
       <c r="D14">
-        <v>4.8389660000000001E-3</v>
+        <v>4.8577789999999996E-3</v>
       </c>
       <c r="E14">
-        <v>4.8389660000000001E-3</v>
+        <v>4.8577789999999996E-3</v>
       </c>
       <c r="F14">
         <v>0</v>
@@ -18781,7 +18781,7 @@
         <v>0</v>
       </c>
       <c r="H14">
-        <v>1.4516897999999999E-2</v>
+        <v>1.4573336999999997E-2</v>
       </c>
     </row>
     <row r="15" spans="1:8">

</xml_diff>

<commit_message>
updated AVL, BAADTbVT, BHNVFEAL, BNVFE, SYFAFE for freight calibration
</commit_message>
<xml_diff>
--- a/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
+++ b/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Olivia Ashmoore\Documents\EPS_Models by Region\United States\us-eps\InputData\trans\BHNVFEAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28AC5378-ED77-42E3-8839-619BE7FF2F86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D77C2360-6206-45AD-A5B2-FB9CD1B26A33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3693,181 +3693,181 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="68"/>
                 <c:pt idx="9" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="10" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="11" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="12" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="13" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="14" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="15" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="16" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="17" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="18" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="19" formatCode="0.00E+00">
-                  <c:v>9.8438896867039508E-4</c:v>
+                  <c:v>1.0506747874471361E-3</c:v>
                 </c:pt>
                 <c:pt idx="20" formatCode="0.00E+00">
-                  <c:v>9.8557760355181558E-4</c:v>
+                  <c:v>1.0488504305659774E-3</c:v>
                 </c:pt>
                 <c:pt idx="21" formatCode="0.00E+00">
-                  <c:v>9.8676623843323608E-4</c:v>
+                  <c:v>1.0470260736848186E-3</c:v>
                 </c:pt>
                 <c:pt idx="22" formatCode="0.00E+00">
-                  <c:v>9.8795487331465657E-4</c:v>
+                  <c:v>1.04520171680366E-3</c:v>
                 </c:pt>
                 <c:pt idx="23" formatCode="0.00E+00">
-                  <c:v>9.8914350819607707E-4</c:v>
+                  <c:v>1.0433773599225014E-3</c:v>
                 </c:pt>
                 <c:pt idx="24" formatCode="0.00E+00">
-                  <c:v>9.9033214307749757E-4</c:v>
+                  <c:v>1.0415530030413428E-3</c:v>
                 </c:pt>
                 <c:pt idx="25" formatCode="0.00E+00">
-                  <c:v>9.9152077795891806E-4</c:v>
+                  <c:v>1.0397286461601841E-3</c:v>
                 </c:pt>
                 <c:pt idx="26" formatCode="0.00E+00">
-                  <c:v>9.9270941284033856E-4</c:v>
+                  <c:v>1.0379042892790255E-3</c:v>
                 </c:pt>
                 <c:pt idx="27" formatCode="0.00E+00">
-                  <c:v>9.9389804772175906E-4</c:v>
+                  <c:v>1.0360799323978669E-3</c:v>
                 </c:pt>
                 <c:pt idx="28" formatCode="0.00E+00">
-                  <c:v>9.9508668260317955E-4</c:v>
+                  <c:v>1.0342555755167083E-3</c:v>
                 </c:pt>
                 <c:pt idx="29" formatCode="0.00E+00">
-                  <c:v>9.9627531748460005E-4</c:v>
+                  <c:v>1.0324312186355497E-3</c:v>
                 </c:pt>
                 <c:pt idx="30" formatCode="0.00E+00">
-                  <c:v>9.9746395236602055E-4</c:v>
+                  <c:v>1.030606861754391E-3</c:v>
                 </c:pt>
                 <c:pt idx="31" formatCode="0.00E+00">
-                  <c:v>9.9865258724744104E-4</c:v>
+                  <c:v>1.0287825048732324E-3</c:v>
                 </c:pt>
                 <c:pt idx="32" formatCode="0.00E+00">
-                  <c:v>9.9984122212886154E-4</c:v>
+                  <c:v>1.0269581479920738E-3</c:v>
                 </c:pt>
                 <c:pt idx="33" formatCode="0.00E+00">
-                  <c:v>1.001029857010282E-3</c:v>
+                  <c:v>1.0251337911109152E-3</c:v>
                 </c:pt>
                 <c:pt idx="34" formatCode="0.00E+00">
-                  <c:v>1.0022184918917025E-3</c:v>
+                  <c:v>1.0233094342297566E-3</c:v>
                 </c:pt>
                 <c:pt idx="35" formatCode="0.00E+00">
-                  <c:v>1.003407126773123E-3</c:v>
+                  <c:v>1.0214850773485979E-3</c:v>
                 </c:pt>
                 <c:pt idx="36" formatCode="0.00E+00">
-                  <c:v>1.0045957616545435E-3</c:v>
+                  <c:v>1.0196607204674393E-3</c:v>
                 </c:pt>
                 <c:pt idx="37" formatCode="0.00E+00">
-                  <c:v>1.005784396535964E-3</c:v>
+                  <c:v>1.0178363635862807E-3</c:v>
                 </c:pt>
                 <c:pt idx="38" formatCode="0.00E+00">
-                  <c:v>1.0069730314173845E-3</c:v>
+                  <c:v>1.0160120067051221E-3</c:v>
                 </c:pt>
                 <c:pt idx="39" formatCode="0.00E+00">
-                  <c:v>1.008161666298805E-3</c:v>
+                  <c:v>1.0141876498239635E-3</c:v>
                 </c:pt>
                 <c:pt idx="40" formatCode="0.00E+00">
                   <c:v>1.0105389360616456E-3</c:v>
                 </c:pt>
                 <c:pt idx="41" formatCode="0.00E+00">
-                  <c:v>1.0071619859986915E-3</c:v>
+                  <c:v>1.0754660288918199E-3</c:v>
                 </c:pt>
                 <c:pt idx="42" formatCode="0.00E+00">
-                  <c:v>1.0297946332597221E-3</c:v>
+                  <c:v>1.0997832463414735E-3</c:v>
                 </c:pt>
                 <c:pt idx="43" formatCode="0.00E+00">
-                  <c:v>1.0542694402792506E-3</c:v>
+                  <c:v>1.1259180725970582E-3</c:v>
                 </c:pt>
                 <c:pt idx="44" formatCode="0.00E+00">
-                  <c:v>1.0790300186124084E-3</c:v>
+                  <c:v>1.1522254447480843E-3</c:v>
                 </c:pt>
                 <c:pt idx="45" formatCode="0.00E+00">
-                  <c:v>1.1024390235193078E-3</c:v>
+                  <c:v>1.1772174874709175E-3</c:v>
                 </c:pt>
                 <c:pt idx="46" formatCode="0.00E+00">
-                  <c:v>1.1250162796311157E-3</c:v>
+                  <c:v>1.2013234498187955E-3</c:v>
                 </c:pt>
                 <c:pt idx="47" formatCode="0.00E+00">
-                  <c:v>1.1437364311026228E-3</c:v>
+                  <c:v>1.2212854897622565E-3</c:v>
                 </c:pt>
                 <c:pt idx="48" formatCode="0.00E+00">
-                  <c:v>1.1601755544794832E-3</c:v>
+                  <c:v>1.238809319858962E-3</c:v>
                 </c:pt>
                 <c:pt idx="49" formatCode="0.00E+00">
-                  <c:v>1.1731175422229271E-3</c:v>
+                  <c:v>1.25258619281297E-3</c:v>
                 </c:pt>
                 <c:pt idx="50" formatCode="0.00E+00">
-                  <c:v>1.1829709958873008E-3</c:v>
+                  <c:v>1.2631583509478295E-3</c:v>
                 </c:pt>
                 <c:pt idx="51" formatCode="0.00E+00">
-                  <c:v>1.1904376346468411E-3</c:v>
+                  <c:v>1.271115521969759E-3</c:v>
                 </c:pt>
                 <c:pt idx="52" formatCode="0.00E+00">
-                  <c:v>1.1951266350083583E-3</c:v>
+                  <c:v>1.2761007035628495E-3</c:v>
                 </c:pt>
                 <c:pt idx="53" formatCode="0.00E+00">
-                  <c:v>1.1954817554531098E-3</c:v>
+                  <c:v>1.2764716537304337E-3</c:v>
                 </c:pt>
                 <c:pt idx="54" formatCode="0.00E+00">
-                  <c:v>1.1956768733474535E-3</c:v>
+                  <c:v>1.2767311778020512E-3</c:v>
                 </c:pt>
                 <c:pt idx="55" formatCode="0.00E+00">
-                  <c:v>1.1953490811620006E-3</c:v>
+                  <c:v>1.276353645502216E-3</c:v>
                 </c:pt>
                 <c:pt idx="56" formatCode="0.00E+00">
-                  <c:v>1.195614135891968E-3</c:v>
+                  <c:v>1.2766760132650891E-3</c:v>
                 </c:pt>
                 <c:pt idx="57" formatCode="0.00E+00">
-                  <c:v>1.1955621240436263E-3</c:v>
+                  <c:v>1.2766818118101673E-3</c:v>
                 </c:pt>
                 <c:pt idx="58" formatCode="0.00E+00">
-                  <c:v>1.1954516355974314E-3</c:v>
+                  <c:v>1.2766739759384397E-3</c:v>
                 </c:pt>
                 <c:pt idx="59" formatCode="0.00E+00">
-                  <c:v>1.1954450239217949E-3</c:v>
+                  <c:v>1.2766888640947222E-3</c:v>
                 </c:pt>
                 <c:pt idx="60" formatCode="0.00E+00">
-                  <c:v>1.1950872588067892E-3</c:v>
+                  <c:v>1.2763212049932639E-3</c:v>
                 </c:pt>
                 <c:pt idx="61" formatCode="0.00E+00">
-                  <c:v>1.1949745664687152E-3</c:v>
+                  <c:v>1.276284062961275E-3</c:v>
                 </c:pt>
                 <c:pt idx="62" formatCode="0.00E+00">
-                  <c:v>1.1948443899217356E-3</c:v>
+                  <c:v>1.2762870405925318E-3</c:v>
                 </c:pt>
                 <c:pt idx="63" formatCode="0.00E+00">
-                  <c:v>1.1946410441643772E-3</c:v>
+                  <c:v>1.2761892489133713E-3</c:v>
                 </c:pt>
                 <c:pt idx="64" formatCode="0.00E+00">
-                  <c:v>1.1944371107025177E-3</c:v>
+                  <c:v>1.2761347112461472E-3</c:v>
                 </c:pt>
                 <c:pt idx="65" formatCode="0.00E+00">
-                  <c:v>1.193589934664274E-3</c:v>
+                  <c:v>1.2753821541254299E-3</c:v>
                 </c:pt>
                 <c:pt idx="66" formatCode="0.00E+00">
-                  <c:v>1.1933357524675759E-3</c:v>
+                  <c:v>1.2752958028189919E-3</c:v>
                 </c:pt>
                 <c:pt idx="67" formatCode="0.00E+00">
-                  <c:v>1.1931159509841881E-3</c:v>
+                  <c:v>1.2752821684021858E-3</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -4234,148 +4234,148 @@
                   <c:v>7.8040477200267344E-4</c:v>
                 </c:pt>
                 <c:pt idx="20" formatCode="0.00E+00">
-                  <c:v>7.8134709903309753E-4</c:v>
+                  <c:v>7.7904970301948082E-4</c:v>
                 </c:pt>
                 <c:pt idx="21" formatCode="0.00E+00">
-                  <c:v>7.8228942606352163E-4</c:v>
+                  <c:v>7.7769463403628821E-4</c:v>
                 </c:pt>
                 <c:pt idx="22" formatCode="0.00E+00">
-                  <c:v>7.8323175309394572E-4</c:v>
+                  <c:v>7.7633956505309559E-4</c:v>
                 </c:pt>
                 <c:pt idx="23" formatCode="0.00E+00">
-                  <c:v>7.8417408012436982E-4</c:v>
+                  <c:v>7.7498449606990298E-4</c:v>
                 </c:pt>
                 <c:pt idx="24" formatCode="0.00E+00">
-                  <c:v>7.8511640715479391E-4</c:v>
+                  <c:v>7.7362942708671036E-4</c:v>
                 </c:pt>
                 <c:pt idx="25" formatCode="0.00E+00">
-                  <c:v>7.8605873418521801E-4</c:v>
+                  <c:v>7.7227435810351774E-4</c:v>
                 </c:pt>
                 <c:pt idx="26" formatCode="0.00E+00">
-                  <c:v>7.870010612156421E-4</c:v>
+                  <c:v>7.7091928912032513E-4</c:v>
                 </c:pt>
                 <c:pt idx="27" formatCode="0.00E+00">
-                  <c:v>7.879433882460662E-4</c:v>
+                  <c:v>7.6956422013713251E-4</c:v>
                 </c:pt>
                 <c:pt idx="28" formatCode="0.00E+00">
-                  <c:v>7.8888571527649029E-4</c:v>
+                  <c:v>7.682091511539399E-4</c:v>
                 </c:pt>
                 <c:pt idx="29" formatCode="0.00E+00">
-                  <c:v>7.8982804230691439E-4</c:v>
+                  <c:v>7.6685408217074728E-4</c:v>
                 </c:pt>
                 <c:pt idx="30" formatCode="0.00E+00">
-                  <c:v>7.9077036933733848E-4</c:v>
+                  <c:v>7.6549901318755467E-4</c:v>
                 </c:pt>
                 <c:pt idx="31" formatCode="0.00E+00">
-                  <c:v>7.9171269636776258E-4</c:v>
+                  <c:v>7.6414394420436205E-4</c:v>
                 </c:pt>
                 <c:pt idx="32" formatCode="0.00E+00">
-                  <c:v>7.9265502339818667E-4</c:v>
+                  <c:v>7.6278887522116944E-4</c:v>
                 </c:pt>
                 <c:pt idx="33" formatCode="0.00E+00">
-                  <c:v>7.9359735042861077E-4</c:v>
+                  <c:v>7.6143380623797682E-4</c:v>
                 </c:pt>
                 <c:pt idx="34" formatCode="0.00E+00">
-                  <c:v>7.9453967745903486E-4</c:v>
+                  <c:v>7.6007873725478421E-4</c:v>
                 </c:pt>
                 <c:pt idx="35" formatCode="0.00E+00">
-                  <c:v>7.9548200448945896E-4</c:v>
+                  <c:v>7.5872366827159159E-4</c:v>
                 </c:pt>
                 <c:pt idx="36" formatCode="0.00E+00">
-                  <c:v>7.9642433151988306E-4</c:v>
+                  <c:v>7.5736859928839898E-4</c:v>
                 </c:pt>
                 <c:pt idx="37" formatCode="0.00E+00">
-                  <c:v>7.9736665855030715E-4</c:v>
+                  <c:v>7.5601353030520636E-4</c:v>
                 </c:pt>
                 <c:pt idx="38" formatCode="0.00E+00">
-                  <c:v>7.9830898558073125E-4</c:v>
+                  <c:v>7.5465846132201375E-4</c:v>
                 </c:pt>
                 <c:pt idx="39" formatCode="0.00E+00">
-                  <c:v>7.9925131261115534E-4</c:v>
+                  <c:v>7.5330339233882113E-4</c:v>
                 </c:pt>
                 <c:pt idx="40" formatCode="0.00E+00">
-                  <c:v>8.0113596667200321E-4</c:v>
+                  <c:v>7.5059325437243547E-4</c:v>
                 </c:pt>
                 <c:pt idx="41" formatCode="0.00E+00">
-                  <c:v>7.9845878516365723E-4</c:v>
+                  <c:v>7.9881884585164282E-4</c:v>
                 </c:pt>
                 <c:pt idx="42" formatCode="0.00E+00">
-                  <c:v>8.1640151561645602E-4</c:v>
+                  <c:v>8.1688083112650234E-4</c:v>
                 </c:pt>
                 <c:pt idx="43" formatCode="0.00E+00">
-                  <c:v>8.3580467513954908E-4</c:v>
+                  <c:v>8.3629287314844459E-4</c:v>
                 </c:pt>
                 <c:pt idx="44" formatCode="0.00E+00">
-                  <c:v>8.5543438870170133E-4</c:v>
+                  <c:v>8.5583307627389927E-4</c:v>
                 </c:pt>
                 <c:pt idx="45" formatCode="0.00E+00">
-                  <c:v>8.7399260066729594E-4</c:v>
+                  <c:v>8.7439629834414924E-4</c:v>
                 </c:pt>
                 <c:pt idx="46" formatCode="0.00E+00">
-                  <c:v>8.9189141807499185E-4</c:v>
+                  <c:v>8.923013706603032E-4</c:v>
                 </c:pt>
                 <c:pt idx="47" formatCode="0.00E+00">
-                  <c:v>9.0673239659663221E-4</c:v>
+                  <c:v>9.0712848121526056E-4</c:v>
                 </c:pt>
                 <c:pt idx="48" formatCode="0.00E+00">
-                  <c:v>9.1976501961370109E-4</c:v>
+                  <c:v>9.2014457410586974E-4</c:v>
                 </c:pt>
                 <c:pt idx="49" formatCode="0.00E+00">
-                  <c:v>9.3002518029777076E-4</c:v>
+                  <c:v>9.3037755725635133E-4</c:v>
                 </c:pt>
                 <c:pt idx="50" formatCode="0.00E+00">
-                  <c:v>9.3783681015661687E-4</c:v>
+                  <c:v>9.3823018944795273E-4</c:v>
                 </c:pt>
                 <c:pt idx="51" formatCode="0.00E+00">
-                  <c:v>9.4375621874836048E-4</c:v>
+                  <c:v>9.4414049995634845E-4</c:v>
                 </c:pt>
                 <c:pt idx="52" formatCode="0.00E+00">
-                  <c:v>9.4747356867254048E-4</c:v>
+                  <c:v>9.4784331984983853E-4</c:v>
                 </c:pt>
                 <c:pt idx="53" formatCode="0.00E+00">
-                  <c:v>9.4775510137814763E-4</c:v>
+                  <c:v>9.4811884876174954E-4</c:v>
                 </c:pt>
                 <c:pt idx="54" formatCode="0.00E+00">
-                  <c:v>9.4790978711792664E-4</c:v>
+                  <c:v>9.4831161423624246E-4</c:v>
                 </c:pt>
                 <c:pt idx="55" formatCode="0.00E+00">
-                  <c:v>9.4764991973430679E-4</c:v>
+                  <c:v>9.4803119634490583E-4</c:v>
                 </c:pt>
                 <c:pt idx="56" formatCode="0.00E+00">
-                  <c:v>9.4786005006153686E-4</c:v>
+                  <c:v>9.4827063993248566E-4</c:v>
                 </c:pt>
                 <c:pt idx="57" formatCode="0.00E+00">
-                  <c:v>9.4781881606162595E-4</c:v>
+                  <c:v>9.4827494689055081E-4</c:v>
                 </c:pt>
                 <c:pt idx="58" formatCode="0.00E+00">
-                  <c:v>9.4773122293187136E-4</c:v>
+                  <c:v>9.4826912667694905E-4</c:v>
                 </c:pt>
                 <c:pt idx="59" formatCode="0.00E+00">
-                  <c:v>9.4772598132171319E-4</c:v>
+                  <c:v>9.4828018508279254E-4</c:v>
                 </c:pt>
                 <c:pt idx="60" formatCode="0.00E+00">
-                  <c:v>9.4744235197204304E-4</c:v>
+                  <c:v>9.4800710066059429E-4</c:v>
                 </c:pt>
                 <c:pt idx="61" formatCode="0.00E+00">
-                  <c:v>9.4735301163890236E-4</c:v>
+                  <c:v>9.4797951284812155E-4</c:v>
                 </c:pt>
                 <c:pt idx="62" formatCode="0.00E+00">
-                  <c:v>9.4724981015889911E-4</c:v>
+                  <c:v>9.4798172452929027E-4</c:v>
                 </c:pt>
                 <c:pt idx="63" formatCode="0.00E+00">
-                  <c:v>9.4708860152647881E-4</c:v>
+                  <c:v>9.4790908826353931E-4</c:v>
                 </c:pt>
                 <c:pt idx="64" formatCode="0.00E+00">
-                  <c:v>9.4692692697315531E-4</c:v>
+                  <c:v>9.4786857957687037E-4</c:v>
                 </c:pt>
                 <c:pt idx="65" formatCode="0.00E+00">
-                  <c:v>9.4625530199155417E-4</c:v>
+                  <c:v>9.4730960626254984E-4</c:v>
                 </c:pt>
                 <c:pt idx="66" formatCode="0.00E+00">
-                  <c:v>9.4605379120102872E-4</c:v>
+                  <c:v>9.4724546750865753E-4</c:v>
                 </c:pt>
                 <c:pt idx="67" formatCode="0.00E+00">
-                  <c:v>9.4587953678332564E-4</c:v>
+                  <c:v>9.472353403369903E-4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8494,123 +8494,123 @@
         <v>5</v>
       </c>
       <c r="B5" s="4">
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="1"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="D5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="F5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="G5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="H5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="I5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="J5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="K5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="L5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="N5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="O5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="P5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="Q5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="R5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="S5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="T5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="U5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="V5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="W5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="X5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="Y5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="Z5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="AA5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="AB5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="AC5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="AD5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="AE5" s="4">
         <f t="shared" si="0"/>
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="AG5" s="4"/>
       <c r="AH5" s="4"/>
@@ -16544,85 +16544,85 @@
         <v>1.0105389360616456E-3</v>
       </c>
       <c r="G10" s="4">
-        <v>1.0071619859986915E-3</v>
+        <v>1.0754660288918199E-3</v>
       </c>
       <c r="H10" s="4">
-        <v>1.0297946332597221E-3</v>
+        <v>1.0997832463414735E-3</v>
       </c>
       <c r="I10" s="4">
-        <v>1.0542694402792506E-3</v>
+        <v>1.1259180725970582E-3</v>
       </c>
       <c r="J10" s="4">
-        <v>1.0790300186124084E-3</v>
+        <v>1.1522254447480843E-3</v>
       </c>
       <c r="K10" s="4">
-        <v>1.1024390235193078E-3</v>
+        <v>1.1772174874709175E-3</v>
       </c>
       <c r="L10" s="4">
-        <v>1.1250162796311157E-3</v>
+        <v>1.2013234498187955E-3</v>
       </c>
       <c r="M10" s="4">
-        <v>1.1437364311026228E-3</v>
+        <v>1.2212854897622565E-3</v>
       </c>
       <c r="N10" s="4">
-        <v>1.1601755544794832E-3</v>
+        <v>1.238809319858962E-3</v>
       </c>
       <c r="O10" s="4">
-        <v>1.1731175422229271E-3</v>
+        <v>1.25258619281297E-3</v>
       </c>
       <c r="P10" s="4">
-        <v>1.1829709958873008E-3</v>
+        <v>1.2631583509478295E-3</v>
       </c>
       <c r="Q10" s="4">
-        <v>1.1904376346468411E-3</v>
+        <v>1.271115521969759E-3</v>
       </c>
       <c r="R10" s="4">
-        <v>1.1951266350083583E-3</v>
+        <v>1.2761007035628495E-3</v>
       </c>
       <c r="S10" s="4">
-        <v>1.1954817554531098E-3</v>
+        <v>1.2764716537304337E-3</v>
       </c>
       <c r="T10" s="4">
-        <v>1.1956768733474535E-3</v>
+        <v>1.2767311778020512E-3</v>
       </c>
       <c r="U10" s="4">
-        <v>1.1953490811620006E-3</v>
+        <v>1.276353645502216E-3</v>
       </c>
       <c r="V10" s="4">
-        <v>1.195614135891968E-3</v>
+        <v>1.2766760132650891E-3</v>
       </c>
       <c r="W10" s="4">
-        <v>1.1955621240436263E-3</v>
+        <v>1.2766818118101673E-3</v>
       </c>
       <c r="X10" s="4">
-        <v>1.1954516355974314E-3</v>
+        <v>1.2766739759384397E-3</v>
       </c>
       <c r="Y10" s="4">
-        <v>1.1954450239217949E-3</v>
+        <v>1.2766888640947222E-3</v>
       </c>
       <c r="Z10" s="4">
-        <v>1.1950872588067892E-3</v>
+        <v>1.2763212049932639E-3</v>
       </c>
       <c r="AA10" s="4">
-        <v>1.1949745664687152E-3</v>
+        <v>1.276284062961275E-3</v>
       </c>
       <c r="AB10" s="4">
-        <v>1.1948443899217356E-3</v>
+        <v>1.2762870405925318E-3</v>
       </c>
       <c r="AC10" s="4">
-        <v>1.1946410441643772E-3</v>
+        <v>1.2761892489133713E-3</v>
       </c>
       <c r="AD10" s="4">
-        <v>1.1944371107025177E-3</v>
+        <v>1.2761347112461472E-3</v>
       </c>
       <c r="AE10" s="4">
-        <v>1.193589934664274E-3</v>
+        <v>1.2753821541254299E-3</v>
       </c>
       <c r="AF10" s="4">
-        <v>1.1933357524675759E-3</v>
+        <v>1.2752958028189919E-3</v>
       </c>
       <c r="AG10" s="4">
-        <v>1.1931159509841881E-3</v>
+        <v>1.2752821684021858E-3</v>
       </c>
       <c r="AH10" s="4"/>
       <c r="AI10" s="4"/>
@@ -16646,88 +16646,88 @@
         <v>7.9651924557390657E-4</v>
       </c>
       <c r="F11" s="4">
-        <v>8.0113596667200321E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="G11" s="4">
-        <v>7.9845878516365723E-4</v>
+        <v>7.9881884585164282E-4</v>
       </c>
       <c r="H11" s="4">
-        <v>8.1640151561645602E-4</v>
+        <v>8.1688083112650234E-4</v>
       </c>
       <c r="I11" s="4">
-        <v>8.3580467513954908E-4</v>
+        <v>8.3629287314844459E-4</v>
       </c>
       <c r="J11" s="4">
-        <v>8.5543438870170133E-4</v>
+        <v>8.5583307627389927E-4</v>
       </c>
       <c r="K11" s="4">
-        <v>8.7399260066729594E-4</v>
+        <v>8.7439629834414924E-4</v>
       </c>
       <c r="L11" s="4">
-        <v>8.9189141807499185E-4</v>
+        <v>8.923013706603032E-4</v>
       </c>
       <c r="M11" s="4">
-        <v>9.0673239659663221E-4</v>
+        <v>9.0712848121526056E-4</v>
       </c>
       <c r="N11" s="4">
-        <v>9.1976501961370109E-4</v>
+        <v>9.2014457410586974E-4</v>
       </c>
       <c r="O11" s="4">
-        <v>9.3002518029777076E-4</v>
+        <v>9.3037755725635133E-4</v>
       </c>
       <c r="P11" s="4">
-        <v>9.3783681015661687E-4</v>
+        <v>9.3823018944795273E-4</v>
       </c>
       <c r="Q11" s="4">
-        <v>9.4375621874836048E-4</v>
+        <v>9.4414049995634845E-4</v>
       </c>
       <c r="R11" s="4">
-        <v>9.4747356867254048E-4</v>
+        <v>9.4784331984983853E-4</v>
       </c>
       <c r="S11" s="4">
-        <v>9.4775510137814763E-4</v>
+        <v>9.4811884876174954E-4</v>
       </c>
       <c r="T11" s="4">
-        <v>9.4790978711792664E-4</v>
+        <v>9.4831161423624246E-4</v>
       </c>
       <c r="U11" s="4">
-        <v>9.4764991973430679E-4</v>
+        <v>9.4803119634490583E-4</v>
       </c>
       <c r="V11" s="4">
-        <v>9.4786005006153686E-4</v>
+        <v>9.4827063993248566E-4</v>
       </c>
       <c r="W11" s="4">
-        <v>9.4781881606162595E-4</v>
+        <v>9.4827494689055081E-4</v>
       </c>
       <c r="X11" s="4">
-        <v>9.4773122293187136E-4</v>
+        <v>9.4826912667694905E-4</v>
       </c>
       <c r="Y11" s="4">
-        <v>9.4772598132171319E-4</v>
+        <v>9.4828018508279254E-4</v>
       </c>
       <c r="Z11" s="4">
-        <v>9.4744235197204304E-4</v>
+        <v>9.4800710066059429E-4</v>
       </c>
       <c r="AA11" s="4">
-        <v>9.4735301163890236E-4</v>
+        <v>9.4797951284812155E-4</v>
       </c>
       <c r="AB11" s="4">
-        <v>9.4724981015889911E-4</v>
+        <v>9.4798172452929027E-4</v>
       </c>
       <c r="AC11" s="4">
-        <v>9.4708860152647881E-4</v>
+        <v>9.4790908826353931E-4</v>
       </c>
       <c r="AD11" s="4">
-        <v>9.4692692697315531E-4</v>
+        <v>9.4786857957687037E-4</v>
       </c>
       <c r="AE11" s="4">
-        <v>9.4625530199155417E-4</v>
+        <v>9.4730960626254984E-4</v>
       </c>
       <c r="AF11" s="4">
-        <v>9.4605379120102872E-4</v>
+        <v>9.4724546750865753E-4</v>
       </c>
       <c r="AG11" s="4">
-        <v>9.4587953678332564E-4</v>
+        <v>9.472353403369903E-4</v>
       </c>
       <c r="AH11" s="4"/>
       <c r="AI11" s="4"/>
@@ -18694,7 +18694,7 @@
         <v>7.5502679371825096E-4</v>
       </c>
       <c r="E11">
-        <v>7.2905101417222013E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="F11">
         <v>0</v>
@@ -19851,127 +19851,127 @@
       <c r="K4" s="9"/>
       <c r="L4" s="4">
         <f>L5/M5*M4</f>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="M4" s="4">
         <f t="shared" ref="M4:AI4" si="1">M5/N5*N4</f>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="N4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="O4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="P4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="Q4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="R4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="S4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="T4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="U4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="V4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8438896867039508E-4</v>
+        <v>1.0506747874471361E-3</v>
       </c>
       <c r="W4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8557760355181558E-4</v>
+        <v>1.0488504305659774E-3</v>
       </c>
       <c r="X4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8676623843323608E-4</v>
+        <v>1.0470260736848186E-3</v>
       </c>
       <c r="Y4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8795487331465657E-4</v>
+        <v>1.04520171680366E-3</v>
       </c>
       <c r="Z4" s="4">
         <f t="shared" si="1"/>
-        <v>9.8914350819607707E-4</v>
+        <v>1.0433773599225014E-3</v>
       </c>
       <c r="AA4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9033214307749757E-4</v>
+        <v>1.0415530030413428E-3</v>
       </c>
       <c r="AB4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9152077795891806E-4</v>
+        <v>1.0397286461601841E-3</v>
       </c>
       <c r="AC4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9270941284033856E-4</v>
+        <v>1.0379042892790255E-3</v>
       </c>
       <c r="AD4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9389804772175906E-4</v>
+        <v>1.0360799323978669E-3</v>
       </c>
       <c r="AE4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9508668260317955E-4</v>
+        <v>1.0342555755167083E-3</v>
       </c>
       <c r="AF4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9627531748460005E-4</v>
+        <v>1.0324312186355497E-3</v>
       </c>
       <c r="AG4" s="4">
         <f>AG5/AH5*AH4</f>
-        <v>9.9746395236602055E-4</v>
+        <v>1.030606861754391E-3</v>
       </c>
       <c r="AH4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9865258724744104E-4</v>
+        <v>1.0287825048732324E-3</v>
       </c>
       <c r="AI4" s="4">
         <f t="shared" si="1"/>
-        <v>9.9984122212886154E-4</v>
+        <v>1.0269581479920738E-3</v>
       </c>
       <c r="AJ4" s="4">
         <f>AJ5/AK5*AK4</f>
-        <v>1.001029857010282E-3</v>
+        <v>1.0251337911109152E-3</v>
       </c>
       <c r="AK4" s="19">
         <f>AK5/AL5*AL4</f>
-        <v>1.0022184918917025E-3</v>
+        <v>1.0233094342297566E-3</v>
       </c>
       <c r="AL4" s="19">
         <f>AL5/AM5*AM4</f>
-        <v>1.003407126773123E-3</v>
+        <v>1.0214850773485979E-3</v>
       </c>
       <c r="AM4" s="19">
         <f>AM5/AN5*AN4</f>
-        <v>1.0045957616545435E-3</v>
+        <v>1.0196607204674393E-3</v>
       </c>
       <c r="AN4" s="19">
         <f t="shared" ref="AN4:AQ4" si="2">AN5/AO5*AO4</f>
-        <v>1.005784396535964E-3</v>
+        <v>1.0178363635862807E-3</v>
       </c>
       <c r="AO4" s="19">
         <f t="shared" si="2"/>
-        <v>1.0069730314173845E-3</v>
+        <v>1.0160120067051221E-3</v>
       </c>
       <c r="AP4" s="19">
         <f t="shared" si="2"/>
-        <v>1.008161666298805E-3</v>
+        <v>1.0141876498239635E-3</v>
       </c>
       <c r="AQ4" s="19">
         <f t="shared" si="2"/>
@@ -19979,111 +19979,111 @@
       </c>
       <c r="AR4" s="10">
         <f>BNVFE!G10</f>
-        <v>1.0071619859986915E-3</v>
+        <v>1.0754660288918199E-3</v>
       </c>
       <c r="AS4" s="10">
         <f>BNVFE!H10</f>
-        <v>1.0297946332597221E-3</v>
+        <v>1.0997832463414735E-3</v>
       </c>
       <c r="AT4" s="10">
         <f>BNVFE!I10</f>
-        <v>1.0542694402792506E-3</v>
+        <v>1.1259180725970582E-3</v>
       </c>
       <c r="AU4" s="10">
         <f>BNVFE!J10</f>
-        <v>1.0790300186124084E-3</v>
+        <v>1.1522254447480843E-3</v>
       </c>
       <c r="AV4" s="10">
         <f>BNVFE!K10</f>
-        <v>1.1024390235193078E-3</v>
+        <v>1.1772174874709175E-3</v>
       </c>
       <c r="AW4" s="10">
         <f>BNVFE!L10</f>
-        <v>1.1250162796311157E-3</v>
+        <v>1.2013234498187955E-3</v>
       </c>
       <c r="AX4" s="10">
         <f>BNVFE!M10</f>
-        <v>1.1437364311026228E-3</v>
+        <v>1.2212854897622565E-3</v>
       </c>
       <c r="AY4" s="10">
         <f>BNVFE!N10</f>
-        <v>1.1601755544794832E-3</v>
+        <v>1.238809319858962E-3</v>
       </c>
       <c r="AZ4" s="10">
         <f>BNVFE!O10</f>
-        <v>1.1731175422229271E-3</v>
+        <v>1.25258619281297E-3</v>
       </c>
       <c r="BA4" s="10">
         <f>BNVFE!P10</f>
-        <v>1.1829709958873008E-3</v>
+        <v>1.2631583509478295E-3</v>
       </c>
       <c r="BB4" s="10">
         <f>BNVFE!Q10</f>
-        <v>1.1904376346468411E-3</v>
+        <v>1.271115521969759E-3</v>
       </c>
       <c r="BC4" s="10">
         <f>BNVFE!R10</f>
-        <v>1.1951266350083583E-3</v>
+        <v>1.2761007035628495E-3</v>
       </c>
       <c r="BD4" s="10">
         <f>BNVFE!S10</f>
-        <v>1.1954817554531098E-3</v>
+        <v>1.2764716537304337E-3</v>
       </c>
       <c r="BE4" s="10">
         <f>BNVFE!T10</f>
-        <v>1.1956768733474535E-3</v>
+        <v>1.2767311778020512E-3</v>
       </c>
       <c r="BF4" s="10">
         <f>BNVFE!U10</f>
-        <v>1.1953490811620006E-3</v>
+        <v>1.276353645502216E-3</v>
       </c>
       <c r="BG4" s="10">
         <f>BNVFE!V10</f>
-        <v>1.195614135891968E-3</v>
+        <v>1.2766760132650891E-3</v>
       </c>
       <c r="BH4" s="10">
         <f>BNVFE!W10</f>
-        <v>1.1955621240436263E-3</v>
+        <v>1.2766818118101673E-3</v>
       </c>
       <c r="BI4" s="10">
         <f>BNVFE!X10</f>
-        <v>1.1954516355974314E-3</v>
+        <v>1.2766739759384397E-3</v>
       </c>
       <c r="BJ4" s="10">
         <f>BNVFE!Y10</f>
-        <v>1.1954450239217949E-3</v>
+        <v>1.2766888640947222E-3</v>
       </c>
       <c r="BK4" s="10">
         <f>BNVFE!Z10</f>
-        <v>1.1950872588067892E-3</v>
+        <v>1.2763212049932639E-3</v>
       </c>
       <c r="BL4" s="10">
         <f>BNVFE!AA10</f>
-        <v>1.1949745664687152E-3</v>
+        <v>1.276284062961275E-3</v>
       </c>
       <c r="BM4" s="10">
         <f>BNVFE!AB10</f>
-        <v>1.1948443899217356E-3</v>
+        <v>1.2762870405925318E-3</v>
       </c>
       <c r="BN4" s="10">
         <f>BNVFE!AC10</f>
-        <v>1.1946410441643772E-3</v>
+        <v>1.2761892489133713E-3</v>
       </c>
       <c r="BO4" s="10">
         <f>BNVFE!AD10</f>
-        <v>1.1944371107025177E-3</v>
+        <v>1.2761347112461472E-3</v>
       </c>
       <c r="BP4" s="10">
         <f>BNVFE!AE10</f>
-        <v>1.193589934664274E-3</v>
+        <v>1.2753821541254299E-3</v>
       </c>
       <c r="BQ4" s="10">
         <f>BNVFE!AF10</f>
-        <v>1.1933357524675759E-3</v>
+        <v>1.2752958028189919E-3</v>
       </c>
       <c r="BR4" s="10">
         <f>BNVFE!AG10</f>
-        <v>1.1931159509841881E-3</v>
+        <v>1.2752821684021858E-3</v>
       </c>
       <c r="BS4" s="10"/>
       <c r="BT4" s="4"/>
@@ -20150,195 +20150,195 @@
       </c>
       <c r="W5" s="4">
         <f>($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+V5</f>
-        <v>7.8134709903309753E-4</v>
+        <v>7.7904970301948082E-4</v>
       </c>
       <c r="X5" s="4">
         <f t="shared" ref="X5:AN5" si="4">($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+W5</f>
-        <v>7.8228942606352163E-4</v>
+        <v>7.7769463403628821E-4</v>
       </c>
       <c r="Y5" s="4">
         <f t="shared" si="4"/>
-        <v>7.8323175309394572E-4</v>
+        <v>7.7633956505309559E-4</v>
       </c>
       <c r="Z5" s="4">
         <f t="shared" si="4"/>
-        <v>7.8417408012436982E-4</v>
+        <v>7.7498449606990298E-4</v>
       </c>
       <c r="AA5" s="4">
         <f t="shared" si="4"/>
-        <v>7.8511640715479391E-4</v>
+        <v>7.7362942708671036E-4</v>
       </c>
       <c r="AB5" s="4">
         <f t="shared" si="4"/>
-        <v>7.8605873418521801E-4</v>
+        <v>7.7227435810351774E-4</v>
       </c>
       <c r="AC5" s="4">
         <f t="shared" si="4"/>
-        <v>7.870010612156421E-4</v>
+        <v>7.7091928912032513E-4</v>
       </c>
       <c r="AD5" s="4">
         <f t="shared" si="4"/>
-        <v>7.879433882460662E-4</v>
+        <v>7.6956422013713251E-4</v>
       </c>
       <c r="AE5" s="4">
         <f t="shared" si="4"/>
-        <v>7.8888571527649029E-4</v>
+        <v>7.682091511539399E-4</v>
       </c>
       <c r="AF5" s="4">
         <f t="shared" si="4"/>
-        <v>7.8982804230691439E-4</v>
+        <v>7.6685408217074728E-4</v>
       </c>
       <c r="AG5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9077036933733848E-4</v>
+        <v>7.6549901318755467E-4</v>
       </c>
       <c r="AH5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9171269636776258E-4</v>
+        <v>7.6414394420436205E-4</v>
       </c>
       <c r="AI5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9265502339818667E-4</v>
+        <v>7.6278887522116944E-4</v>
       </c>
       <c r="AJ5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9359735042861077E-4</v>
+        <v>7.6143380623797682E-4</v>
       </c>
       <c r="AK5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9453967745903486E-4</v>
+        <v>7.6007873725478421E-4</v>
       </c>
       <c r="AL5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9548200448945896E-4</v>
+        <v>7.5872366827159159E-4</v>
       </c>
       <c r="AM5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9642433151988306E-4</v>
+        <v>7.5736859928839898E-4</v>
       </c>
       <c r="AN5" s="4">
         <f t="shared" si="4"/>
-        <v>7.9736665855030715E-4</v>
+        <v>7.5601353030520636E-4</v>
       </c>
       <c r="AO5" s="4">
         <f>($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+AN5</f>
-        <v>7.9830898558073125E-4</v>
+        <v>7.5465846132201375E-4</v>
       </c>
       <c r="AP5" s="4">
         <f>($AQ$5-$V$5)/COUNT($V$1:$AQ$1)+AO5</f>
-        <v>7.9925131261115534E-4</v>
+        <v>7.5330339233882113E-4</v>
       </c>
       <c r="AQ5" s="28">
         <f>BNVFE!F11</f>
-        <v>8.0113596667200321E-4</v>
+        <v>7.5059325437243547E-4</v>
       </c>
       <c r="AR5" s="10">
         <f>BNVFE!G11</f>
-        <v>7.9845878516365723E-4</v>
+        <v>7.9881884585164282E-4</v>
       </c>
       <c r="AS5" s="10">
         <f>BNVFE!H11</f>
-        <v>8.1640151561645602E-4</v>
+        <v>8.1688083112650234E-4</v>
       </c>
       <c r="AT5" s="10">
         <f>BNVFE!I11</f>
-        <v>8.3580467513954908E-4</v>
+        <v>8.3629287314844459E-4</v>
       </c>
       <c r="AU5" s="10">
         <f>BNVFE!J11</f>
-        <v>8.5543438870170133E-4</v>
+        <v>8.5583307627389927E-4</v>
       </c>
       <c r="AV5" s="10">
         <f>BNVFE!K11</f>
-        <v>8.7399260066729594E-4</v>
+        <v>8.7439629834414924E-4</v>
       </c>
       <c r="AW5" s="10">
         <f>BNVFE!L11</f>
-        <v>8.9189141807499185E-4</v>
+        <v>8.923013706603032E-4</v>
       </c>
       <c r="AX5" s="10">
         <f>BNVFE!M11</f>
-        <v>9.0673239659663221E-4</v>
+        <v>9.0712848121526056E-4</v>
       </c>
       <c r="AY5" s="10">
         <f>BNVFE!N11</f>
-        <v>9.1976501961370109E-4</v>
+        <v>9.2014457410586974E-4</v>
       </c>
       <c r="AZ5" s="10">
         <f>BNVFE!O11</f>
-        <v>9.3002518029777076E-4</v>
+        <v>9.3037755725635133E-4</v>
       </c>
       <c r="BA5" s="10">
         <f>BNVFE!P11</f>
-        <v>9.3783681015661687E-4</v>
+        <v>9.3823018944795273E-4</v>
       </c>
       <c r="BB5" s="10">
         <f>BNVFE!Q11</f>
-        <v>9.4375621874836048E-4</v>
+        <v>9.4414049995634845E-4</v>
       </c>
       <c r="BC5" s="10">
         <f>BNVFE!R11</f>
-        <v>9.4747356867254048E-4</v>
+        <v>9.4784331984983853E-4</v>
       </c>
       <c r="BD5" s="10">
         <f>BNVFE!S11</f>
-        <v>9.4775510137814763E-4</v>
+        <v>9.4811884876174954E-4</v>
       </c>
       <c r="BE5" s="10">
         <f>BNVFE!T11</f>
-        <v>9.4790978711792664E-4</v>
+        <v>9.4831161423624246E-4</v>
       </c>
       <c r="BF5" s="10">
         <f>BNVFE!U11</f>
-        <v>9.4764991973430679E-4</v>
+        <v>9.4803119634490583E-4</v>
       </c>
       <c r="BG5" s="10">
         <f>BNVFE!V11</f>
-        <v>9.4786005006153686E-4</v>
+        <v>9.4827063993248566E-4</v>
       </c>
       <c r="BH5" s="10">
         <f>BNVFE!W11</f>
-        <v>9.4781881606162595E-4</v>
+        <v>9.4827494689055081E-4</v>
       </c>
       <c r="BI5" s="10">
         <f>BNVFE!X11</f>
-        <v>9.4773122293187136E-4</v>
+        <v>9.4826912667694905E-4</v>
       </c>
       <c r="BJ5" s="10">
         <f>BNVFE!Y11</f>
-        <v>9.4772598132171319E-4</v>
+        <v>9.4828018508279254E-4</v>
       </c>
       <c r="BK5" s="10">
         <f>BNVFE!Z11</f>
-        <v>9.4744235197204304E-4</v>
+        <v>9.4800710066059429E-4</v>
       </c>
       <c r="BL5" s="10">
         <f>BNVFE!AA11</f>
-        <v>9.4735301163890236E-4</v>
+        <v>9.4797951284812155E-4</v>
       </c>
       <c r="BM5" s="10">
         <f>BNVFE!AB11</f>
-        <v>9.4724981015889911E-4</v>
+        <v>9.4798172452929027E-4</v>
       </c>
       <c r="BN5" s="10">
         <f>BNVFE!AC11</f>
-        <v>9.4708860152647881E-4</v>
+        <v>9.4790908826353931E-4</v>
       </c>
       <c r="BO5" s="10">
         <f>BNVFE!AD11</f>
-        <v>9.4692692697315531E-4</v>
+        <v>9.4786857957687037E-4</v>
       </c>
       <c r="BP5" s="10">
         <f>BNVFE!AE11</f>
-        <v>9.4625530199155417E-4</v>
+        <v>9.4730960626254984E-4</v>
       </c>
       <c r="BQ5" s="10">
         <f>BNVFE!AF11</f>
-        <v>9.4605379120102872E-4</v>
+        <v>9.4724546750865753E-4</v>
       </c>
       <c r="BR5" s="10">
         <f>BNVFE!AG11</f>
-        <v>9.4587953678332564E-4</v>
+        <v>9.472353403369903E-4</v>
       </c>
       <c r="BS5" s="10"/>
       <c r="BT5" s="4"/>

</xml_diff>

<commit_message>
calibrate aircraft BAADTbVT, BCDTRTSY, BHNVFEAL, BNVFE, SYFAFE, SYVBT
</commit_message>
<xml_diff>
--- a/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
+++ b/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\trans\BHNVFEAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F78C7657-5FEF-479C-AB5D-811D6ABB0F6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65B1C6E-2B31-47A2-A24A-04186B1BE671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4710,169 +4710,169 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="70"/>
                 <c:pt idx="13" formatCode="0.00E+00">
-                  <c:v>3.3000958546164708E-4</c:v>
+                  <c:v>2.290338125160345E-4</c:v>
                 </c:pt>
                 <c:pt idx="14" formatCode="0.00E+00">
-                  <c:v>3.3397333498517805E-4</c:v>
+                  <c:v>2.3241910879234773E-4</c:v>
                 </c:pt>
                 <c:pt idx="15" formatCode="0.00E+00">
-                  <c:v>3.3793708450870902E-4</c:v>
+                  <c:v>2.3580440506866095E-4</c:v>
                 </c:pt>
                 <c:pt idx="16" formatCode="0.00E+00">
-                  <c:v>3.4190083403223999E-4</c:v>
+                  <c:v>2.3918970134497418E-4</c:v>
                 </c:pt>
                 <c:pt idx="17" formatCode="0.00E+00">
-                  <c:v>3.4586458355577096E-4</c:v>
+                  <c:v>2.4257499762128654E-4</c:v>
                 </c:pt>
                 <c:pt idx="18" formatCode="0.00E+00">
-                  <c:v>3.4982833307930193E-4</c:v>
+                  <c:v>2.4596029389759976E-4</c:v>
                 </c:pt>
                 <c:pt idx="19" formatCode="0.00E+00">
-                  <c:v>3.537920826028329E-4</c:v>
+                  <c:v>2.4934559017391299E-4</c:v>
                 </c:pt>
                 <c:pt idx="20" formatCode="0.00E+00">
-                  <c:v>3.5775583212636387E-4</c:v>
+                  <c:v>2.5273088645022621E-4</c:v>
                 </c:pt>
                 <c:pt idx="21" formatCode="0.00E+00">
-                  <c:v>3.6171958164989484E-4</c:v>
+                  <c:v>2.5611618272653944E-4</c:v>
                 </c:pt>
                 <c:pt idx="22" formatCode="0.00E+00">
-                  <c:v>3.6568333117342582E-4</c:v>
+                  <c:v>2.595014790028518E-4</c:v>
                 </c:pt>
                 <c:pt idx="23" formatCode="0.00E+00">
-                  <c:v>3.6964708069695679E-4</c:v>
+                  <c:v>2.6288677527916502E-4</c:v>
                 </c:pt>
                 <c:pt idx="24" formatCode="0.00E+00">
-                  <c:v>3.7361083022048776E-4</c:v>
+                  <c:v>2.6627207155547825E-4</c:v>
                 </c:pt>
                 <c:pt idx="25" formatCode="0.00E+00">
-                  <c:v>3.7757457974401873E-4</c:v>
+                  <c:v>2.6965736783179147E-4</c:v>
                 </c:pt>
                 <c:pt idx="26" formatCode="0.00E+00">
-                  <c:v>3.815383292675497E-4</c:v>
+                  <c:v>2.7304266410810383E-4</c:v>
                 </c:pt>
                 <c:pt idx="27" formatCode="0.00E+00">
-                  <c:v>3.8550207879108067E-4</c:v>
+                  <c:v>2.7642796038441705E-4</c:v>
                 </c:pt>
                 <c:pt idx="28" formatCode="0.00E+00">
-                  <c:v>3.8946582831461164E-4</c:v>
+                  <c:v>2.7981325666073028E-4</c:v>
                 </c:pt>
                 <c:pt idx="29" formatCode="0.00E+00">
-                  <c:v>3.9342957783814261E-4</c:v>
+                  <c:v>2.831985529370435E-4</c:v>
                 </c:pt>
                 <c:pt idx="30" formatCode="0.00E+00">
-                  <c:v>3.9739332736167358E-4</c:v>
+                  <c:v>2.8658384921335586E-4</c:v>
                 </c:pt>
                 <c:pt idx="31" formatCode="0.00E+00">
-                  <c:v>4.0135707688520629E-4</c:v>
+                  <c:v>2.8996914548966909E-4</c:v>
                 </c:pt>
                 <c:pt idx="32" formatCode="0.00E+00">
-                  <c:v>4.0532082640873726E-4</c:v>
+                  <c:v>2.9335444176598231E-4</c:v>
                 </c:pt>
                 <c:pt idx="33" formatCode="0.00E+00">
-                  <c:v>4.0928457593226823E-4</c:v>
+                  <c:v>2.9673973804229554E-4</c:v>
                 </c:pt>
                 <c:pt idx="34" formatCode="0.00E+00">
-                  <c:v>4.132483254557992E-4</c:v>
+                  <c:v>3.001250343186079E-4</c:v>
                 </c:pt>
                 <c:pt idx="35" formatCode="0.00E+00">
-                  <c:v>4.1721207497933017E-4</c:v>
+                  <c:v>3.0351033059492112E-4</c:v>
                 </c:pt>
                 <c:pt idx="36" formatCode="0.00E+00">
-                  <c:v>4.2117582450286115E-4</c:v>
+                  <c:v>3.0689562687123435E-4</c:v>
                 </c:pt>
                 <c:pt idx="37" formatCode="0.00E+00">
-                  <c:v>4.2513957402639212E-4</c:v>
+                  <c:v>3.1028092314754757E-4</c:v>
                 </c:pt>
                 <c:pt idx="38" formatCode="0.00E+00">
-                  <c:v>4.2910332354992309E-4</c:v>
+                  <c:v>3.1366621942385993E-4</c:v>
                 </c:pt>
                 <c:pt idx="39" formatCode="0.00E+00">
-                  <c:v>4.3306707307345406E-4</c:v>
+                  <c:v>3.1705151570017315E-4</c:v>
                 </c:pt>
                 <c:pt idx="40" formatCode="0.00E+00">
-                  <c:v>4.3956547255263602E-4</c:v>
+                  <c:v>3.0464933987873528E-4</c:v>
                 </c:pt>
                 <c:pt idx="41" formatCode="0.00E+00">
-                  <c:v>4.4366680476890972E-4</c:v>
+                  <c:v>3.0464933987873528E-4</c:v>
                 </c:pt>
                 <c:pt idx="42" formatCode="0.00E+00">
-                  <c:v>4.4597245060431232E-4</c:v>
+                  <c:v>3.3408269543052564E-4</c:v>
                 </c:pt>
                 <c:pt idx="43" formatCode="0.00E+00">
-                  <c:v>4.4931411605150481E-4</c:v>
+                  <c:v>3.3665348546582375E-4</c:v>
                 </c:pt>
                 <c:pt idx="44" formatCode="0.00E+00">
-                  <c:v>4.5288823478004158E-4</c:v>
+                  <c:v>3.3935581504087849E-4</c:v>
                 </c:pt>
                 <c:pt idx="45" formatCode="0.00E+00">
-                  <c:v>4.5662840926832999E-4</c:v>
+                  <c:v>3.4216015354620157E-4</c:v>
                 </c:pt>
                 <c:pt idx="46" formatCode="0.00E+00">
-                  <c:v>4.6040875969022651E-4</c:v>
+                  <c:v>3.4502111275582734E-4</c:v>
                 </c:pt>
                 <c:pt idx="47" formatCode="0.00E+00">
-                  <c:v>4.6419842254086203E-4</c:v>
+                  <c:v>3.4790902074721106E-4</c:v>
                 </c:pt>
                 <c:pt idx="48" formatCode="0.00E+00">
-                  <c:v>4.6802171784268048E-4</c:v>
+                  <c:v>3.5081980617662339E-4</c:v>
                 </c:pt>
                 <c:pt idx="49" formatCode="0.00E+00">
-                  <c:v>4.718495549789862E-4</c:v>
+                  <c:v>3.5375247221412683E-4</c:v>
                 </c:pt>
                 <c:pt idx="50" formatCode="0.00E+00">
-                  <c:v>4.7569706545502331E-4</c:v>
+                  <c:v>3.5670603348759934E-4</c:v>
                 </c:pt>
                 <c:pt idx="51" formatCode="0.00E+00">
-                  <c:v>4.7956228574948121E-4</c:v>
+                  <c:v>3.5968007751568736E-4</c:v>
                 </c:pt>
                 <c:pt idx="52" formatCode="0.00E+00">
-                  <c:v>4.8344561142611898E-4</c:v>
+                  <c:v>3.626744897202374E-4</c:v>
                 </c:pt>
                 <c:pt idx="53" formatCode="0.00E+00">
-                  <c:v>4.8740041976327717E-4</c:v>
+                  <c:v>3.656928831323635E-4</c:v>
                 </c:pt>
                 <c:pt idx="54" formatCode="0.00E+00">
-                  <c:v>4.9138744510057676E-4</c:v>
+                  <c:v>3.6873385989859042E-4</c:v>
                 </c:pt>
                 <c:pt idx="55" formatCode="0.00E+00">
-                  <c:v>4.9540734035651132E-4</c:v>
+                  <c:v>3.7179596105709373E-4</c:v>
                 </c:pt>
                 <c:pt idx="56" formatCode="0.00E+00">
-                  <c:v>4.9946276009751292E-4</c:v>
+                  <c:v>3.7487939284855035E-4</c:v>
                 </c:pt>
                 <c:pt idx="57" formatCode="0.00E+00">
-                  <c:v>5.0354741343006288E-4</c:v>
+                  <c:v>3.7798229146832611E-4</c:v>
                 </c:pt>
                 <c:pt idx="58" formatCode="0.00E+00">
-                  <c:v>5.076679534506399E-4</c:v>
+                  <c:v>3.8110333926765313E-4</c:v>
                 </c:pt>
                 <c:pt idx="59" formatCode="0.00E+00">
-                  <c:v>5.1181172688478038E-4</c:v>
+                  <c:v>3.8424184495833714E-4</c:v>
                 </c:pt>
                 <c:pt idx="60" formatCode="0.00E+00">
-                  <c:v>5.1597913882790009E-4</c:v>
+                  <c:v>3.8739917202040771E-4</c:v>
                 </c:pt>
                 <c:pt idx="61" formatCode="0.00E+00">
-                  <c:v>5.2017698058550235E-4</c:v>
+                  <c:v>3.9057663428336076E-4</c:v>
                 </c:pt>
                 <c:pt idx="62" formatCode="0.00E+00">
-                  <c:v>5.2440413218790766E-4</c:v>
+                  <c:v>3.937746365900064E-4</c:v>
                 </c:pt>
                 <c:pt idx="63" formatCode="0.00E+00">
-                  <c:v>5.2866665576887042E-4</c:v>
+                  <c:v>3.9699374037329777E-4</c:v>
                 </c:pt>
                 <c:pt idx="64" formatCode="0.00E+00">
-                  <c:v>5.3296936481509794E-4</c:v>
+                  <c:v>4.0023428554842422E-4</c:v>
                 </c:pt>
                 <c:pt idx="65" formatCode="0.00E+00">
-                  <c:v>5.3730424796901105E-4</c:v>
+                  <c:v>4.0349549298394053E-4</c:v>
                 </c:pt>
                 <c:pt idx="66" formatCode="0.00E+00">
-                  <c:v>5.4167698609809006E-4</c:v>
+                  <c:v>4.067774772580003E-4</c:v>
                 </c:pt>
                 <c:pt idx="67" formatCode="0.00E+00">
-                  <c:v>5.4607888156546253E-4</c:v>
+                  <c:v>4.1007787424136491E-4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -5206,169 +5206,169 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="70"/>
                 <c:pt idx="13" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="14" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="15" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="16" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="17" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="18" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="19" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="20" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="21" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="22" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="23" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="24" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="25" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="26" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="27" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="28" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="29" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="30" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="31" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="32" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="33" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="34" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="35" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="36" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="37" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="38" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="39" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="40" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="41" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>9.3239985476639982E-5</c:v>
                 </c:pt>
                 <c:pt idx="42" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0224826248544657E-4</c:v>
                 </c:pt>
                 <c:pt idx="43" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0303507011696843E-4</c:v>
                 </c:pt>
                 <c:pt idx="44" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0386213631193046E-4</c:v>
                 </c:pt>
                 <c:pt idx="45" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0472042302810055E-4</c:v>
                 </c:pt>
                 <c:pt idx="46" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0559603889275644E-4</c:v>
                 </c:pt>
                 <c:pt idx="47" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0647990261385189E-4</c:v>
                 </c:pt>
                 <c:pt idx="48" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0737076812917535E-4</c:v>
                 </c:pt>
                 <c:pt idx="49" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0826833035220035E-4</c:v>
                 </c:pt>
                 <c:pt idx="50" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.0917228770314212E-4</c:v>
                 </c:pt>
                 <c:pt idx="51" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1008251393930003E-4</c:v>
                 </c:pt>
                 <c:pt idx="52" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1099897399325733E-4</c:v>
                 </c:pt>
                 <c:pt idx="53" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1192277365755811E-4</c:v>
                 </c:pt>
                 <c:pt idx="54" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1285348510971702E-4</c:v>
                 </c:pt>
                 <c:pt idx="55" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1379066182462636E-4</c:v>
                 </c:pt>
                 <c:pt idx="56" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1473436692363647E-4</c:v>
                 </c:pt>
                 <c:pt idx="57" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.156840299767668E-4</c:v>
                 </c:pt>
                 <c:pt idx="58" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1663924770872375E-4</c:v>
                 </c:pt>
                 <c:pt idx="59" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1759980854609242E-4</c:v>
                 </c:pt>
                 <c:pt idx="60" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1856612979113317E-4</c:v>
                 </c:pt>
                 <c:pt idx="61" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.1953861355022565E-4</c:v>
                 </c:pt>
                 <c:pt idx="62" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.2051738372824274E-4</c:v>
                 </c:pt>
                 <c:pt idx="63" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.2150261215552689E-4</c:v>
                 </c:pt>
                 <c:pt idx="64" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.2249440286541473E-4</c:v>
                 </c:pt>
                 <c:pt idx="65" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.2349251739947177E-4</c:v>
                 </c:pt>
                 <c:pt idx="66" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.2449699082511483E-4</c:v>
                 </c:pt>
                 <c:pt idx="67" formatCode="0.00E+00">
-                  <c:v>1.8223851973329149E-4</c:v>
+                  <c:v>1.2550709958464328E-4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9112,123 +9112,123 @@
       </c>
       <c r="B2" s="4">
         <f>B$5/(1-'Other Values'!$B$3)</f>
-        <v>1.0732148425526729E-3</v>
+        <v>7.4687291205413782E-4</v>
       </c>
       <c r="C2" s="4">
         <f>C$5/(1-'Other Values'!$B$3)</f>
-        <v>1.085952251127532E-3</v>
+        <v>7.5775147578839195E-4</v>
       </c>
       <c r="D2" s="4">
         <f>D$5/(1-'Other Values'!$B$3)</f>
-        <v>1.0986896597023912E-3</v>
+        <v>7.6863003952264597E-4</v>
       </c>
       <c r="E2" s="4">
         <f>E$5/(1-'Other Values'!$B$3)</f>
-        <v>1.1114270682772503E-3</v>
+        <v>7.7950860325689728E-4</v>
       </c>
       <c r="F2" s="4">
         <f>F$5/(1-'Other Values'!$B$3)</f>
-        <v>1.1241644768521094E-3</v>
+        <v>7.9038716699115141E-4</v>
       </c>
       <c r="G2" s="4">
         <f>G$5/(1-'Other Values'!$B$3)</f>
-        <v>1.1369018854269686E-3</v>
+        <v>8.0126573072540543E-4</v>
       </c>
       <c r="H2" s="4">
         <f>H$5/(1-'Other Values'!$B$3)</f>
-        <v>1.1496392940018279E-3</v>
+        <v>8.1214429445965956E-4</v>
       </c>
       <c r="I2" s="4">
         <f>I$5/(1-'Other Values'!$B$3)</f>
-        <v>1.1623767025766871E-3</v>
+        <v>8.2302285819391358E-4</v>
       </c>
       <c r="J2" s="4">
         <f>J$5/(1-'Other Values'!$B$3)</f>
-        <v>1.1751141111515462E-3</v>
+        <v>8.3390142192816489E-4</v>
       </c>
       <c r="K2" s="4">
         <f>K$5/(1-'Other Values'!$B$3)</f>
-        <v>1.1878515197264053E-3</v>
+        <v>8.4477998566241902E-4</v>
       </c>
       <c r="L2" s="4">
         <f>L$5/(1-'Other Values'!$B$3)</f>
-        <v>1.2005889283012645E-3</v>
+        <v>8.5565854939667304E-4</v>
       </c>
       <c r="M2" s="4">
         <f>M$5/(1-'Other Values'!$B$3)</f>
-        <v>1.2133263368761238E-3</v>
+        <v>8.6653711313092717E-4</v>
       </c>
       <c r="N2" s="4">
         <f>N$5/(1-'Other Values'!$B$3)</f>
-        <v>1.226063745450983E-3</v>
+        <v>8.7741567686517848E-4</v>
       </c>
       <c r="O2" s="4">
         <f>O$5/(1-'Other Values'!$B$3)</f>
-        <v>1.2388011540258421E-3</v>
+        <v>8.882942405994325E-4</v>
       </c>
       <c r="P2" s="4">
         <f>P$5/(1-'Other Values'!$B$3)</f>
-        <v>1.2515385626007012E-3</v>
+        <v>8.9917280433368663E-4</v>
       </c>
       <c r="Q2" s="4">
         <f>Q$5/(1-'Other Values'!$B$3)</f>
-        <v>1.2642759711755604E-3</v>
+        <v>9.1005136806794065E-4</v>
       </c>
       <c r="R2" s="4">
         <f>R$5/(1-'Other Values'!$B$3)</f>
-        <v>1.2770133797504195E-3</v>
+        <v>9.2092993180219196E-4</v>
       </c>
       <c r="S2" s="4">
         <f>S$5/(1-'Other Values'!$B$3)</f>
-        <v>1.2897507883252843E-3</v>
+        <v>9.3180849553644609E-4</v>
       </c>
       <c r="T2" s="4">
         <f>T$5/(1-'Other Values'!$B$3)</f>
-        <v>1.3024881969001436E-3</v>
+        <v>9.4268705927070011E-4</v>
       </c>
       <c r="U2" s="4">
         <f>U$5/(1-'Other Values'!$B$3)</f>
-        <v>1.3152256054750028E-3</v>
+        <v>9.5356562300495423E-4</v>
       </c>
       <c r="V2" s="4">
         <f>V$5/(1-'Other Values'!$B$3)</f>
-        <v>1.3279630140498619E-3</v>
+        <v>9.6444418673920554E-4</v>
       </c>
       <c r="W2" s="4">
         <f>W$5/(1-'Other Values'!$B$3)</f>
-        <v>1.340700422624721E-3</v>
+        <v>9.7532275047345956E-4</v>
       </c>
       <c r="X2" s="4">
         <f>X$5/(1-'Other Values'!$B$3)</f>
-        <v>1.3534378311995802E-3</v>
+        <v>9.8620131420771358E-4</v>
       </c>
       <c r="Y2" s="4">
         <f>Y$5/(1-'Other Values'!$B$3)</f>
-        <v>1.3661752397744393E-3</v>
+        <v>9.9707987794196771E-4</v>
       </c>
       <c r="Z2" s="4">
         <f>Z$5/(1-'Other Values'!$B$3)</f>
-        <v>1.3789126483492987E-3</v>
+        <v>1.007958441676219E-3</v>
       </c>
       <c r="AA2" s="4">
         <f>AA$5/(1-'Other Values'!$B$3)</f>
-        <v>1.3916500569241578E-3</v>
+        <v>1.0188370054104732E-3</v>
       </c>
       <c r="AB2" s="4">
         <f>AB$5/(1-'Other Values'!$B$3)</f>
-        <v>1.412532498853853E-3</v>
+        <v>9.7898292792220369E-4</v>
       </c>
       <c r="AC2" s="4">
         <f>AC$5/(1-'Other Values'!$B$3)</f>
-        <v>1.4257120259228021E-3</v>
+        <v>9.7898292792220369E-4</v>
       </c>
       <c r="AD2" s="4">
         <f>AD$5/(1-'Other Values'!$B$3)</f>
-        <v>1.4331211603446675E-3</v>
+        <v>1.0735662695704627E-3</v>
       </c>
       <c r="AE2" s="4">
         <f>AE$5/(1-'Other Values'!$B$3)</f>
-        <v>1.4438595175160014E-3</v>
+        <v>1.0818274381547478E-3</v>
       </c>
       <c r="AG2" s="4"/>
       <c r="AH2" s="4"/>
@@ -9429,123 +9429,123 @@
       </c>
       <c r="B5">
         <f>Extrapolations!Q6</f>
-        <v>3.3397333498517805E-4</v>
+        <v>2.3241910879234773E-4</v>
       </c>
       <c r="C5" s="4">
         <f>Extrapolations!R6</f>
-        <v>3.3793708450870902E-4</v>
+        <v>2.3580440506866095E-4</v>
       </c>
       <c r="D5" s="4">
         <f>Extrapolations!S6</f>
-        <v>3.4190083403223999E-4</v>
+        <v>2.3918970134497418E-4</v>
       </c>
       <c r="E5" s="4">
         <f>Extrapolations!T6</f>
-        <v>3.4586458355577096E-4</v>
+        <v>2.4257499762128654E-4</v>
       </c>
       <c r="F5" s="4">
         <f>Extrapolations!U6</f>
-        <v>3.4982833307930193E-4</v>
+        <v>2.4596029389759976E-4</v>
       </c>
       <c r="G5" s="4">
         <f>Extrapolations!V6</f>
-        <v>3.537920826028329E-4</v>
+        <v>2.4934559017391299E-4</v>
       </c>
       <c r="H5" s="4">
         <f>Extrapolations!W6</f>
-        <v>3.5775583212636387E-4</v>
+        <v>2.5273088645022621E-4</v>
       </c>
       <c r="I5" s="4">
         <f>Extrapolations!X6</f>
-        <v>3.6171958164989484E-4</v>
+        <v>2.5611618272653944E-4</v>
       </c>
       <c r="J5" s="4">
         <f>Extrapolations!Y6</f>
-        <v>3.6568333117342582E-4</v>
+        <v>2.595014790028518E-4</v>
       </c>
       <c r="K5" s="4">
         <f>Extrapolations!Z6</f>
-        <v>3.6964708069695679E-4</v>
+        <v>2.6288677527916502E-4</v>
       </c>
       <c r="L5" s="4">
         <f>Extrapolations!AA6</f>
-        <v>3.7361083022048776E-4</v>
+        <v>2.6627207155547825E-4</v>
       </c>
       <c r="M5" s="4">
         <f>Extrapolations!AB6</f>
-        <v>3.7757457974401873E-4</v>
+        <v>2.6965736783179147E-4</v>
       </c>
       <c r="N5" s="4">
         <f>Extrapolations!AC6</f>
-        <v>3.815383292675497E-4</v>
+        <v>2.7304266410810383E-4</v>
       </c>
       <c r="O5" s="4">
         <f>Extrapolations!AD6</f>
-        <v>3.8550207879108067E-4</v>
+        <v>2.7642796038441705E-4</v>
       </c>
       <c r="P5" s="4">
         <f>Extrapolations!AE6</f>
-        <v>3.8946582831461164E-4</v>
+        <v>2.7981325666073028E-4</v>
       </c>
       <c r="Q5" s="4">
         <f>Extrapolations!AF6</f>
-        <v>3.9342957783814261E-4</v>
+        <v>2.831985529370435E-4</v>
       </c>
       <c r="R5" s="4">
         <f>Extrapolations!AG6</f>
-        <v>3.9739332736167358E-4</v>
+        <v>2.8658384921335586E-4</v>
       </c>
       <c r="S5" s="4">
         <f>Extrapolations!AH6</f>
-        <v>4.0135707688520629E-4</v>
+        <v>2.8996914548966909E-4</v>
       </c>
       <c r="T5" s="4">
         <f>Extrapolations!AI6</f>
-        <v>4.0532082640873726E-4</v>
+        <v>2.9335444176598231E-4</v>
       </c>
       <c r="U5" s="4">
         <f>Extrapolations!AJ6</f>
-        <v>4.0928457593226823E-4</v>
+        <v>2.9673973804229554E-4</v>
       </c>
       <c r="V5" s="4">
         <f>Extrapolations!AK6</f>
-        <v>4.132483254557992E-4</v>
+        <v>3.001250343186079E-4</v>
       </c>
       <c r="W5" s="4">
         <f>Extrapolations!AL6</f>
-        <v>4.1721207497933017E-4</v>
+        <v>3.0351033059492112E-4</v>
       </c>
       <c r="X5" s="4">
         <f>Extrapolations!AM6</f>
-        <v>4.2117582450286115E-4</v>
+        <v>3.0689562687123435E-4</v>
       </c>
       <c r="Y5" s="4">
         <f>Extrapolations!AN6</f>
-        <v>4.2513957402639212E-4</v>
+        <v>3.1028092314754757E-4</v>
       </c>
       <c r="Z5" s="4">
         <f>Extrapolations!AO6</f>
-        <v>4.2910332354992309E-4</v>
+        <v>3.1366621942385993E-4</v>
       </c>
       <c r="AA5" s="4">
         <f>Extrapolations!AP6</f>
-        <v>4.3306707307345406E-4</v>
+        <v>3.1705151570017315E-4</v>
       </c>
       <c r="AB5" s="4">
         <f>Extrapolations!AQ6</f>
-        <v>4.3956547255263602E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="AC5" s="4">
         <f>Extrapolations!AR6</f>
-        <v>4.4366680476890972E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="AD5" s="4">
         <f>Extrapolations!AS6</f>
-        <v>4.4597245060431232E-4</v>
+        <v>3.3408269543052564E-4</v>
       </c>
       <c r="AE5" s="4">
         <f>Extrapolations!AT6</f>
-        <v>4.4931411605150481E-4</v>
+        <v>3.3665348546582375E-4</v>
       </c>
       <c r="AG5" s="4"/>
       <c r="AH5" s="4"/>
@@ -9746,123 +9746,123 @@
       </c>
       <c r="B8" s="4">
         <f>B$5*Calculations!$B$27</f>
-        <v>1.0019200049555339E-3</v>
+        <v>6.9725732637704308E-4</v>
       </c>
       <c r="C8" s="4">
         <f>C$5*Calculations!$B$27</f>
-        <v>1.0138112535261268E-3</v>
+        <v>7.0741321520598275E-4</v>
       </c>
       <c r="D8" s="4">
         <f>D$5*Calculations!$B$27</f>
-        <v>1.0257025020967198E-3</v>
+        <v>7.1756910403492243E-4</v>
       </c>
       <c r="E8" s="4">
         <f>E$5*Calculations!$B$27</f>
-        <v>1.0375937506673127E-3</v>
+        <v>7.277249928638595E-4</v>
       </c>
       <c r="F8" s="4">
         <f>F$5*Calculations!$B$27</f>
-        <v>1.0494849992379056E-3</v>
+        <v>7.3788088169279918E-4</v>
       </c>
       <c r="G8" s="4">
         <f>G$5*Calculations!$B$27</f>
-        <v>1.0613762478084985E-3</v>
+        <v>7.4803677052173885E-4</v>
       </c>
       <c r="H8" s="4">
         <f>H$5*Calculations!$B$27</f>
-        <v>1.0732674963790914E-3</v>
+        <v>7.5819265935067853E-4</v>
       </c>
       <c r="I8" s="4">
         <f>I$5*Calculations!$B$27</f>
-        <v>1.0851587449496843E-3</v>
+        <v>7.683485481796182E-4</v>
       </c>
       <c r="J8" s="4">
         <f>J$5*Calculations!$B$27</f>
-        <v>1.0970499935202772E-3</v>
+        <v>7.7850443700855528E-4</v>
       </c>
       <c r="K8" s="4">
         <f>K$5*Calculations!$B$27</f>
-        <v>1.1089412420908701E-3</v>
+        <v>7.8866032583749495E-4</v>
       </c>
       <c r="L8" s="4">
         <f>L$5*Calculations!$B$27</f>
-        <v>1.1208324906614631E-3</v>
+        <v>7.9881621466643463E-4</v>
       </c>
       <c r="M8" s="4">
         <f>M$5*Calculations!$B$27</f>
-        <v>1.132723739232056E-3</v>
+        <v>8.089721034953743E-4</v>
       </c>
       <c r="N8" s="4">
         <f>N$5*Calculations!$B$27</f>
-        <v>1.1446149878026489E-3</v>
+        <v>8.1912799232431138E-4</v>
       </c>
       <c r="O8" s="4">
         <f>O$5*Calculations!$B$27</f>
-        <v>1.1565062363732418E-3</v>
+        <v>8.2928388115325105E-4</v>
       </c>
       <c r="P8" s="4">
         <f>P$5*Calculations!$B$27</f>
-        <v>1.1683974849438347E-3</v>
+        <v>8.3943976998219073E-4</v>
       </c>
       <c r="Q8" s="4">
         <f>Q$5*Calculations!$B$27</f>
-        <v>1.1802887335144276E-3</v>
+        <v>8.4959565881113041E-4</v>
       </c>
       <c r="R8" s="4">
         <f>R$5*Calculations!$B$27</f>
-        <v>1.1921799820850205E-3</v>
+        <v>8.5975154764006748E-4</v>
       </c>
       <c r="S8" s="4">
         <f>S$5*Calculations!$B$27</f>
-        <v>1.2040712306556187E-3</v>
+        <v>8.6990743646900715E-4</v>
       </c>
       <c r="T8" s="4">
         <f>T$5*Calculations!$B$27</f>
-        <v>1.2159624792262116E-3</v>
+        <v>8.8006332529794683E-4</v>
       </c>
       <c r="U8" s="4">
         <f>U$5*Calculations!$B$27</f>
-        <v>1.2278537277968045E-3</v>
+        <v>8.9021921412688651E-4</v>
       </c>
       <c r="V8" s="4">
         <f>V$5*Calculations!$B$27</f>
-        <v>1.2397449763673974E-3</v>
+        <v>9.0037510295582358E-4</v>
       </c>
       <c r="W8" s="4">
         <f>W$5*Calculations!$B$27</f>
-        <v>1.2516362249379903E-3</v>
+        <v>9.1053099178476325E-4</v>
       </c>
       <c r="X8" s="4">
         <f>X$5*Calculations!$B$27</f>
-        <v>1.2635274735085832E-3</v>
+        <v>9.2068688061370293E-4</v>
       </c>
       <c r="Y8" s="4">
         <f>Y$5*Calculations!$B$27</f>
-        <v>1.2754187220791761E-3</v>
+        <v>9.3084276944264261E-4</v>
       </c>
       <c r="Z8" s="4">
         <f>Z$5*Calculations!$B$27</f>
-        <v>1.287309970649769E-3</v>
+        <v>9.4099865827157968E-4</v>
       </c>
       <c r="AA8" s="4">
         <f>AA$5*Calculations!$B$27</f>
-        <v>1.299201219220362E-3</v>
+        <v>9.5115454710051936E-4</v>
       </c>
       <c r="AB8" s="4">
         <f>AB$5*Calculations!$B$27</f>
-        <v>1.3186964176579079E-3</v>
+        <v>9.1394801963620568E-4</v>
       </c>
       <c r="AC8" s="4">
         <f>AC$5*Calculations!$B$27</f>
-        <v>1.331000414306729E-3</v>
+        <v>9.1394801963620568E-4</v>
       </c>
       <c r="AD8" s="4">
         <f>AD$5*Calculations!$B$27</f>
-        <v>1.3379173518129367E-3</v>
+        <v>1.0022480862915768E-3</v>
       </c>
       <c r="AE8" s="4">
         <f>AE$5*Calculations!$B$27</f>
-        <v>1.3479423481545143E-3</v>
+        <v>1.0099604563974711E-3</v>
       </c>
       <c r="AG8" s="4"/>
       <c r="AH8" s="4"/>
@@ -9984,123 +9984,123 @@
       </c>
       <c r="B2" s="4">
         <f>B$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="C2" s="4">
         <f>C$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="D2" s="4">
         <f>D$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="E2" s="4">
         <f>E$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="F2" s="4">
         <f>F$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="G2" s="4">
         <f>G$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="H2" s="4">
         <f>H$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="I2" s="4">
         <f>I$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="J2" s="4">
         <f>J$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="K2" s="4">
         <f>K$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="L2" s="4">
         <f>L$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="M2" s="4">
         <f>M$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="N2" s="4">
         <f>N$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="O2" s="4">
         <f>O$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="P2" s="4">
         <f>P$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="Q2" s="4">
         <f>Q$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="R2" s="4">
         <f>R$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="S2" s="4">
         <f>S$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="T2" s="4">
         <f>T$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="U2" s="4">
         <f>U$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="V2" s="4">
         <f>V$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="W2" s="4">
         <f>W$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="X2" s="4">
         <f>X$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="Y2" s="4">
         <f>Y$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="Z2" s="4">
         <f>Z$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="AA2" s="4">
         <f>AA$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="AB2" s="4">
         <f>AB$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="AC2" s="4">
         <f>AC$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="AD2" s="4">
         <f>AD$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>3.2857219852439111E-4</v>
       </c>
       <c r="AE2" s="4">
         <f>AE$5/(1-'Other Values'!$B$3)</f>
-        <v>5.8561886167132651E-4</v>
+        <v>3.3110058489517865E-4</v>
       </c>
       <c r="AG2" s="4"/>
       <c r="AH2" s="4"/>
@@ -10301,123 +10301,123 @@
       </c>
       <c r="B5" s="4">
         <f>Extrapolations!Q7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="C5" s="4">
         <f>Extrapolations!R7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="D5" s="4">
         <f>Extrapolations!S7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="E5" s="4">
         <f>Extrapolations!T7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="F5" s="4">
         <f>Extrapolations!U7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="G5" s="4">
         <f>Extrapolations!V7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="H5" s="4">
         <f>Extrapolations!W7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="I5" s="4">
         <f>Extrapolations!X7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="J5" s="4">
         <f>Extrapolations!Y7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="K5" s="4">
         <f>Extrapolations!Z7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="L5" s="4">
         <f>Extrapolations!AA7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="M5" s="4">
         <f>Extrapolations!AB7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="N5" s="4">
         <f>Extrapolations!AC7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="O5" s="4">
         <f>Extrapolations!AD7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="P5" s="4">
         <f>Extrapolations!AE7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="Q5" s="4">
         <f>Extrapolations!AF7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="R5" s="4">
         <f>Extrapolations!AG7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="S5" s="4">
         <f>Extrapolations!AH7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="T5" s="4">
         <f>Extrapolations!AI7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="U5" s="4">
         <f>Extrapolations!AJ7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="V5" s="4">
         <f>Extrapolations!AK7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="W5" s="4">
         <f>Extrapolations!AL7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="X5" s="4">
         <f>Extrapolations!AM7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="Y5" s="4">
         <f>Extrapolations!AN7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="Z5" s="4">
         <f>Extrapolations!AO7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AA5" s="4">
         <f>Extrapolations!AP7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AB5" s="4">
         <f>Extrapolations!AQ7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AC5" s="4">
         <f>Extrapolations!AR7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AD5" s="4">
         <f>Extrapolations!AS7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0224826248544657E-4</v>
       </c>
       <c r="AE5" s="4">
         <f>Extrapolations!AT7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0303507011696843E-4</v>
       </c>
       <c r="AG5" s="4"/>
       <c r="AH5" s="4"/>
@@ -10618,123 +10618,123 @@
       </c>
       <c r="B8" s="4">
         <f>B$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="C8" s="4">
         <f>C$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="D8" s="4">
         <f>D$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="E8" s="4">
         <f>E$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="F8" s="4">
         <f>F$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="G8" s="4">
         <f>G$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="H8" s="4">
         <f>H$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="I8" s="4">
         <f>I$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="J8" s="4">
         <f>J$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="K8" s="4">
         <f>K$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="L8" s="4">
         <f>L$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="M8" s="4">
         <f>M$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="N8" s="4">
         <f>N$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="O8" s="4">
         <f>O$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="P8" s="4">
         <f>P$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="Q8" s="4">
         <f>Q$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="R8" s="4">
         <f>R$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="S8" s="4">
         <f>S$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="T8" s="4">
         <f>T$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="U8" s="4">
         <f>U$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="V8" s="4">
         <f>V$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="W8" s="4">
         <f>W$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="X8" s="4">
         <f>X$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="Y8" s="4">
         <f>Y$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="Z8" s="4">
         <f>Z$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="AA8" s="4">
         <f>AA$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="AB8" s="4">
         <f>AB$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="AC8" s="4">
         <f>AC$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
       <c r="AD8" s="4">
         <f>AD$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>3.0674478745633968E-4</v>
       </c>
       <c r="AE8" s="4">
         <f>AE$5*Calculations!$B$27</f>
-        <v>5.4671555919987437E-4</v>
+        <v>3.0910521035090526E-4</v>
       </c>
       <c r="AG8" s="4"/>
       <c r="AH8" s="4"/>
@@ -16752,88 +16752,88 @@
         <v>5.7245968727451246E-4</v>
       </c>
       <c r="F12" s="4">
-        <v>4.3956547255263602E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="G12" s="4">
-        <v>4.4366680476890972E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="H12" s="4">
-        <v>4.4597245060431232E-4</v>
+        <v>3.3408269543052564E-4</v>
       </c>
       <c r="I12" s="4">
-        <v>4.4931411605150481E-4</v>
+        <v>3.3665348546582375E-4</v>
       </c>
       <c r="J12" s="4">
-        <v>4.5288823478004158E-4</v>
+        <v>3.3935581504087849E-4</v>
       </c>
       <c r="K12" s="4">
-        <v>4.5662840926832999E-4</v>
+        <v>3.4216015354620157E-4</v>
       </c>
       <c r="L12" s="4">
-        <v>4.6040875969022651E-4</v>
+        <v>3.4502111275582734E-4</v>
       </c>
       <c r="M12" s="4">
-        <v>4.6419842254086203E-4</v>
+        <v>3.4790902074721106E-4</v>
       </c>
       <c r="N12" s="4">
-        <v>4.6802171784268048E-4</v>
+        <v>3.5081980617662339E-4</v>
       </c>
       <c r="O12" s="4">
-        <v>4.718495549789862E-4</v>
+        <v>3.5375247221412683E-4</v>
       </c>
       <c r="P12" s="4">
-        <v>4.7569706545502331E-4</v>
+        <v>3.5670603348759934E-4</v>
       </c>
       <c r="Q12" s="4">
-        <v>4.7956228574948121E-4</v>
+        <v>3.5968007751568736E-4</v>
       </c>
       <c r="R12" s="4">
-        <v>4.8344561142611898E-4</v>
+        <v>3.626744897202374E-4</v>
       </c>
       <c r="S12" s="4">
-        <v>4.8740041976327717E-4</v>
+        <v>3.656928831323635E-4</v>
       </c>
       <c r="T12" s="4">
-        <v>4.9138744510057676E-4</v>
+        <v>3.6873385989859042E-4</v>
       </c>
       <c r="U12" s="4">
-        <v>4.9540734035651132E-4</v>
+        <v>3.7179596105709373E-4</v>
       </c>
       <c r="V12" s="4">
-        <v>4.9946276009751292E-4</v>
+        <v>3.7487939284855035E-4</v>
       </c>
       <c r="W12" s="4">
-        <v>5.0354741343006288E-4</v>
+        <v>3.7798229146832611E-4</v>
       </c>
       <c r="X12" s="4">
-        <v>5.076679534506399E-4</v>
+        <v>3.8110333926765313E-4</v>
       </c>
       <c r="Y12" s="4">
-        <v>5.1181172688478038E-4</v>
+        <v>3.8424184495833714E-4</v>
       </c>
       <c r="Z12" s="4">
-        <v>5.1597913882790009E-4</v>
+        <v>3.8739917202040771E-4</v>
       </c>
       <c r="AA12" s="4">
-        <v>5.2017698058550235E-4</v>
+        <v>3.9057663428336076E-4</v>
       </c>
       <c r="AB12" s="4">
-        <v>5.2440413218790766E-4</v>
+        <v>3.937746365900064E-4</v>
       </c>
       <c r="AC12" s="4">
-        <v>5.2866665576887042E-4</v>
+        <v>3.9699374037329777E-4</v>
       </c>
       <c r="AD12" s="4">
-        <v>5.3296936481509794E-4</v>
+        <v>4.0023428554842422E-4</v>
       </c>
       <c r="AE12" s="4">
-        <v>5.3730424796901105E-4</v>
+        <v>4.0349549298394053E-4</v>
       </c>
       <c r="AF12" s="4">
-        <v>5.4167698609809006E-4</v>
+        <v>4.067774772580003E-4</v>
       </c>
       <c r="AG12" s="4">
-        <v>5.4607888156546253E-4</v>
+        <v>4.1007787424136491E-4</v>
       </c>
       <c r="AH12" s="4"/>
       <c r="AI12" s="4"/>
@@ -16857,88 +16857,88 @@
         <v>4.7951937565239972E-5</v>
       </c>
       <c r="F13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="G13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="H13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0224826248544657E-4</v>
       </c>
       <c r="I13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0303507011696843E-4</v>
       </c>
       <c r="J13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0386213631193046E-4</v>
       </c>
       <c r="K13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0472042302810055E-4</v>
       </c>
       <c r="L13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0559603889275644E-4</v>
       </c>
       <c r="M13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0647990261385189E-4</v>
       </c>
       <c r="N13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0737076812917535E-4</v>
       </c>
       <c r="O13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0826833035220035E-4</v>
       </c>
       <c r="P13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.0917228770314212E-4</v>
       </c>
       <c r="Q13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1008251393930003E-4</v>
       </c>
       <c r="R13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1099897399325733E-4</v>
       </c>
       <c r="S13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1192277365755811E-4</v>
       </c>
       <c r="T13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1285348510971702E-4</v>
       </c>
       <c r="U13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1379066182462636E-4</v>
       </c>
       <c r="V13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1473436692363647E-4</v>
       </c>
       <c r="W13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.156840299767668E-4</v>
       </c>
       <c r="X13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1663924770872375E-4</v>
       </c>
       <c r="Y13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1759980854609242E-4</v>
       </c>
       <c r="Z13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1856612979113317E-4</v>
       </c>
       <c r="AA13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.1953861355022565E-4</v>
       </c>
       <c r="AB13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.2051738372824274E-4</v>
       </c>
       <c r="AC13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.2150261215552689E-4</v>
       </c>
       <c r="AD13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.2249440286541473E-4</v>
       </c>
       <c r="AE13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.2349251739947177E-4</v>
       </c>
       <c r="AF13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.2449699082511483E-4</v>
       </c>
       <c r="AG13" s="4">
-        <v>1.8223851973329149E-4</v>
+        <v>1.2550709958464328E-4</v>
       </c>
       <c r="AH13" s="4"/>
       <c r="AI13" s="4"/>
@@ -18530,16 +18530,16 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <v>1.3074072528197812E-3</v>
+        <v>9.7898292792220369E-4</v>
       </c>
       <c r="C4">
-        <v>4.0685158562424757E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="D4">
-        <v>4.0685158562424757E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="E4">
-        <v>4.0685158562424757E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="F4">
         <v>0</v>
@@ -18548,7 +18548,7 @@
         <v>0</v>
       </c>
       <c r="H4">
-        <v>1.2205547568727424E-3</v>
+        <v>9.1394801963620568E-4</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -18712,16 +18712,16 @@
         <v>7</v>
       </c>
       <c r="B12">
-        <v>5.437858374844844E-4</v>
+        <v>2.9962432880267732E-4</v>
       </c>
       <c r="C12">
-        <v>1.6922051621130835E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="D12">
-        <v>1.6922051621130835E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="E12">
-        <v>1.6922051621130835E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="F12">
         <v>0</v>
@@ -18730,7 +18730,7 @@
         <v>0</v>
       </c>
       <c r="H12">
-        <v>5.0766154863392504E-4</v>
+        <v>2.7971995642991991E-4</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -20365,223 +20365,223 @@
       <c r="O6" s="23"/>
       <c r="P6" s="4">
         <f t="shared" ref="P6:AM6" si="5">TREND($AQ6:$BR6,$AQ$1:$BR$1,P$1)</f>
-        <v>3.3000958546164708E-4</v>
+        <v>2.290338125160345E-4</v>
       </c>
       <c r="Q6" s="4">
         <f>TREND($AQ6:$BR6,$AQ$1:$BR$1,Q$1)</f>
-        <v>3.3397333498517805E-4</v>
+        <v>2.3241910879234773E-4</v>
       </c>
       <c r="R6" s="4">
         <f t="shared" si="5"/>
-        <v>3.3793708450870902E-4</v>
+        <v>2.3580440506866095E-4</v>
       </c>
       <c r="S6" s="4">
         <f t="shared" si="5"/>
-        <v>3.4190083403223999E-4</v>
+        <v>2.3918970134497418E-4</v>
       </c>
       <c r="T6" s="4">
         <f t="shared" si="5"/>
-        <v>3.4586458355577096E-4</v>
+        <v>2.4257499762128654E-4</v>
       </c>
       <c r="U6" s="4">
         <f t="shared" si="5"/>
-        <v>3.4982833307930193E-4</v>
+        <v>2.4596029389759976E-4</v>
       </c>
       <c r="V6" s="4">
         <f t="shared" si="5"/>
-        <v>3.537920826028329E-4</v>
+        <v>2.4934559017391299E-4</v>
       </c>
       <c r="W6" s="4">
         <f t="shared" si="5"/>
-        <v>3.5775583212636387E-4</v>
+        <v>2.5273088645022621E-4</v>
       </c>
       <c r="X6" s="4">
         <f t="shared" si="5"/>
-        <v>3.6171958164989484E-4</v>
+        <v>2.5611618272653944E-4</v>
       </c>
       <c r="Y6" s="4">
         <f t="shared" si="5"/>
-        <v>3.6568333117342582E-4</v>
+        <v>2.595014790028518E-4</v>
       </c>
       <c r="Z6" s="4">
         <f t="shared" si="5"/>
-        <v>3.6964708069695679E-4</v>
+        <v>2.6288677527916502E-4</v>
       </c>
       <c r="AA6" s="4">
         <f t="shared" si="5"/>
-        <v>3.7361083022048776E-4</v>
+        <v>2.6627207155547825E-4</v>
       </c>
       <c r="AB6" s="4">
         <f t="shared" si="5"/>
-        <v>3.7757457974401873E-4</v>
+        <v>2.6965736783179147E-4</v>
       </c>
       <c r="AC6" s="4">
         <f t="shared" si="5"/>
-        <v>3.815383292675497E-4</v>
+        <v>2.7304266410810383E-4</v>
       </c>
       <c r="AD6" s="4">
         <f t="shared" si="5"/>
-        <v>3.8550207879108067E-4</v>
+        <v>2.7642796038441705E-4</v>
       </c>
       <c r="AE6" s="4">
         <f t="shared" si="5"/>
-        <v>3.8946582831461164E-4</v>
+        <v>2.7981325666073028E-4</v>
       </c>
       <c r="AF6" s="4">
         <f t="shared" si="5"/>
-        <v>3.9342957783814261E-4</v>
+        <v>2.831985529370435E-4</v>
       </c>
       <c r="AG6" s="4">
         <f t="shared" si="5"/>
-        <v>3.9739332736167358E-4</v>
+        <v>2.8658384921335586E-4</v>
       </c>
       <c r="AH6" s="4">
         <f t="shared" si="5"/>
-        <v>4.0135707688520629E-4</v>
+        <v>2.8996914548966909E-4</v>
       </c>
       <c r="AI6" s="4">
         <f t="shared" si="5"/>
-        <v>4.0532082640873726E-4</v>
+        <v>2.9335444176598231E-4</v>
       </c>
       <c r="AJ6" s="4">
         <f t="shared" si="5"/>
-        <v>4.0928457593226823E-4</v>
+        <v>2.9673973804229554E-4</v>
       </c>
       <c r="AK6" s="4">
         <f t="shared" si="5"/>
-        <v>4.132483254557992E-4</v>
+        <v>3.001250343186079E-4</v>
       </c>
       <c r="AL6" s="4">
         <f t="shared" si="5"/>
-        <v>4.1721207497933017E-4</v>
+        <v>3.0351033059492112E-4</v>
       </c>
       <c r="AM6" s="4">
         <f t="shared" si="5"/>
-        <v>4.2117582450286115E-4</v>
+        <v>3.0689562687123435E-4</v>
       </c>
       <c r="AN6" s="4">
         <f>TREND($AQ6:$BR6,$AQ$1:$BR$1,AN$1)</f>
-        <v>4.2513957402639212E-4</v>
+        <v>3.1028092314754757E-4</v>
       </c>
       <c r="AO6" s="4">
         <f t="shared" ref="AO6:AP6" si="6">TREND($AQ6:$BR6,$AQ$1:$BR$1,AO$1)</f>
-        <v>4.2910332354992309E-4</v>
+        <v>3.1366621942385993E-4</v>
       </c>
       <c r="AP6" s="4">
         <f t="shared" si="6"/>
-        <v>4.3306707307345406E-4</v>
+        <v>3.1705151570017315E-4</v>
       </c>
       <c r="AQ6" s="26">
         <f>BNVFE!F12</f>
-        <v>4.3956547255263602E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="AR6" s="20">
         <f>BNVFE!G12</f>
-        <v>4.4366680476890972E-4</v>
+        <v>3.0464933987873528E-4</v>
       </c>
       <c r="AS6" s="26">
         <f>BNVFE!H12</f>
-        <v>4.4597245060431232E-4</v>
+        <v>3.3408269543052564E-4</v>
       </c>
       <c r="AT6" s="26">
         <f>BNVFE!I12</f>
-        <v>4.4931411605150481E-4</v>
+        <v>3.3665348546582375E-4</v>
       </c>
       <c r="AU6" s="26">
         <f>BNVFE!J12</f>
-        <v>4.5288823478004158E-4</v>
+        <v>3.3935581504087849E-4</v>
       </c>
       <c r="AV6" s="26">
         <f>BNVFE!K12</f>
-        <v>4.5662840926832999E-4</v>
+        <v>3.4216015354620157E-4</v>
       </c>
       <c r="AW6" s="26">
         <f>BNVFE!L12</f>
-        <v>4.6040875969022651E-4</v>
+        <v>3.4502111275582734E-4</v>
       </c>
       <c r="AX6" s="26">
         <f>BNVFE!M12</f>
-        <v>4.6419842254086203E-4</v>
+        <v>3.4790902074721106E-4</v>
       </c>
       <c r="AY6" s="26">
         <f>BNVFE!N12</f>
-        <v>4.6802171784268048E-4</v>
+        <v>3.5081980617662339E-4</v>
       </c>
       <c r="AZ6" s="26">
         <f>BNVFE!O12</f>
-        <v>4.718495549789862E-4</v>
+        <v>3.5375247221412683E-4</v>
       </c>
       <c r="BA6" s="26">
         <f>BNVFE!P12</f>
-        <v>4.7569706545502331E-4</v>
+        <v>3.5670603348759934E-4</v>
       </c>
       <c r="BB6" s="26">
         <f>BNVFE!Q12</f>
-        <v>4.7956228574948121E-4</v>
+        <v>3.5968007751568736E-4</v>
       </c>
       <c r="BC6" s="26">
         <f>BNVFE!R12</f>
-        <v>4.8344561142611898E-4</v>
+        <v>3.626744897202374E-4</v>
       </c>
       <c r="BD6" s="26">
         <f>BNVFE!S12</f>
-        <v>4.8740041976327717E-4</v>
+        <v>3.656928831323635E-4</v>
       </c>
       <c r="BE6" s="26">
         <f>BNVFE!T12</f>
-        <v>4.9138744510057676E-4</v>
+        <v>3.6873385989859042E-4</v>
       </c>
       <c r="BF6" s="26">
         <f>BNVFE!U12</f>
-        <v>4.9540734035651132E-4</v>
+        <v>3.7179596105709373E-4</v>
       </c>
       <c r="BG6" s="26">
         <f>BNVFE!V12</f>
-        <v>4.9946276009751292E-4</v>
+        <v>3.7487939284855035E-4</v>
       </c>
       <c r="BH6" s="26">
         <f>BNVFE!W12</f>
-        <v>5.0354741343006288E-4</v>
+        <v>3.7798229146832611E-4</v>
       </c>
       <c r="BI6" s="26">
         <f>BNVFE!X12</f>
-        <v>5.076679534506399E-4</v>
+        <v>3.8110333926765313E-4</v>
       </c>
       <c r="BJ6" s="26">
         <f>BNVFE!Y12</f>
-        <v>5.1181172688478038E-4</v>
+        <v>3.8424184495833714E-4</v>
       </c>
       <c r="BK6" s="26">
         <f>BNVFE!Z12</f>
-        <v>5.1597913882790009E-4</v>
+        <v>3.8739917202040771E-4</v>
       </c>
       <c r="BL6" s="26">
         <f>BNVFE!AA12</f>
-        <v>5.2017698058550235E-4</v>
+        <v>3.9057663428336076E-4</v>
       </c>
       <c r="BM6" s="26">
         <f>BNVFE!AB12</f>
-        <v>5.2440413218790766E-4</v>
+        <v>3.937746365900064E-4</v>
       </c>
       <c r="BN6" s="26">
         <f>BNVFE!AC12</f>
-        <v>5.2866665576887042E-4</v>
+        <v>3.9699374037329777E-4</v>
       </c>
       <c r="BO6" s="26">
         <f>BNVFE!AD12</f>
-        <v>5.3296936481509794E-4</v>
+        <v>4.0023428554842422E-4</v>
       </c>
       <c r="BP6" s="26">
         <f>BNVFE!AE12</f>
-        <v>5.3730424796901105E-4</v>
+        <v>4.0349549298394053E-4</v>
       </c>
       <c r="BQ6" s="26">
         <f>BNVFE!AF12</f>
-        <v>5.4167698609809006E-4</v>
+        <v>4.067774772580003E-4</v>
       </c>
       <c r="BR6" s="26">
         <f>BNVFE!AG12</f>
-        <v>5.4607888156546253E-4</v>
+        <v>4.1007787424136491E-4</v>
       </c>
       <c r="BS6" s="26"/>
       <c r="BT6" s="4"/>
@@ -20608,223 +20608,223 @@
       <c r="O7" s="23"/>
       <c r="P7" s="26">
         <f t="shared" ref="P7:AP7" si="7">Q7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="Q7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="R7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="S7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="T7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="U7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="V7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="W7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="X7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="Y7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="Z7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AA7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AB7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AC7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AD7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AE7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AF7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AG7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AH7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AI7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AJ7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AK7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AL7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AM7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AN7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AO7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AP7" s="26">
         <f t="shared" si="7"/>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AQ7" s="26">
         <f>AR7</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AR7" s="20">
         <f>BNVFE!G13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>9.3239985476639982E-5</v>
       </c>
       <c r="AS7" s="26">
         <f>BNVFE!H13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0224826248544657E-4</v>
       </c>
       <c r="AT7" s="26">
         <f>BNVFE!I13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0303507011696843E-4</v>
       </c>
       <c r="AU7" s="26">
         <f>BNVFE!J13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0386213631193046E-4</v>
       </c>
       <c r="AV7" s="26">
         <f>BNVFE!K13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0472042302810055E-4</v>
       </c>
       <c r="AW7" s="26">
         <f>BNVFE!L13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0559603889275644E-4</v>
       </c>
       <c r="AX7" s="26">
         <f>BNVFE!M13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0647990261385189E-4</v>
       </c>
       <c r="AY7" s="26">
         <f>BNVFE!N13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0737076812917535E-4</v>
       </c>
       <c r="AZ7" s="26">
         <f>BNVFE!O13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0826833035220035E-4</v>
       </c>
       <c r="BA7" s="26">
         <f>BNVFE!P13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.0917228770314212E-4</v>
       </c>
       <c r="BB7" s="26">
         <f>BNVFE!Q13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1008251393930003E-4</v>
       </c>
       <c r="BC7" s="26">
         <f>BNVFE!R13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1099897399325733E-4</v>
       </c>
       <c r="BD7" s="26">
         <f>BNVFE!S13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1192277365755811E-4</v>
       </c>
       <c r="BE7" s="26">
         <f>BNVFE!T13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1285348510971702E-4</v>
       </c>
       <c r="BF7" s="26">
         <f>BNVFE!U13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1379066182462636E-4</v>
       </c>
       <c r="BG7" s="26">
         <f>BNVFE!V13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1473436692363647E-4</v>
       </c>
       <c r="BH7" s="26">
         <f>BNVFE!W13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.156840299767668E-4</v>
       </c>
       <c r="BI7" s="26">
         <f>BNVFE!X13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1663924770872375E-4</v>
       </c>
       <c r="BJ7" s="26">
         <f>BNVFE!Y13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1759980854609242E-4</v>
       </c>
       <c r="BK7" s="26">
         <f>BNVFE!Z13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1856612979113317E-4</v>
       </c>
       <c r="BL7" s="26">
         <f>BNVFE!AA13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.1953861355022565E-4</v>
       </c>
       <c r="BM7" s="26">
         <f>BNVFE!AB13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.2051738372824274E-4</v>
       </c>
       <c r="BN7" s="26">
         <f>BNVFE!AC13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.2150261215552689E-4</v>
       </c>
       <c r="BO7" s="26">
         <f>BNVFE!AD13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.2249440286541473E-4</v>
       </c>
       <c r="BP7" s="26">
         <f>BNVFE!AE13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.2349251739947177E-4</v>
       </c>
       <c r="BQ7" s="26">
         <f>BNVFE!AF13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.2449699082511483E-4</v>
       </c>
       <c r="BR7" s="26">
         <f>BNVFE!AG13</f>
-        <v>1.8223851973329149E-4</v>
+        <v>1.2550709958464328E-4</v>
       </c>
       <c r="BS7" s="26"/>
       <c r="BT7" s="4"/>

</xml_diff>

<commit_message>
calibrate freight ldvs BAADTbVT, BhNVFEAL, BNVFE, SYFAFE, SYVBT
</commit_message>
<xml_diff>
--- a/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
+++ b/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\trans\BHNVFEAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B65B1C6E-2B31-47A2-A24A-04186B1BE671}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46122336-199E-4D3F-9ABC-740C7AD03B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="615" yWindow="45" windowWidth="20370" windowHeight="17025" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -3231,136 +3231,136 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="70"/>
                 <c:pt idx="24" formatCode="0.00E+00">
-                  <c:v>5.9551063413003282E-5</c:v>
+                  <c:v>5.8438727152645888E-5</c:v>
                 </c:pt>
                 <c:pt idx="25" formatCode="0.00E+00">
-                  <c:v>6.0878373147410427E-5</c:v>
+                  <c:v>5.9741244470903031E-5</c:v>
                 </c:pt>
                 <c:pt idx="26" formatCode="0.00E+00">
-                  <c:v>6.2205682881817138E-5</c:v>
+                  <c:v>6.1043761789159739E-5</c:v>
                 </c:pt>
                 <c:pt idx="27" formatCode="0.00E+00">
-                  <c:v>6.3532992616224283E-5</c:v>
+                  <c:v>6.2346279107416882E-5</c:v>
                 </c:pt>
                 <c:pt idx="28" formatCode="0.00E+00">
-                  <c:v>6.4860302350631428E-5</c:v>
+                  <c:v>6.3648796425673591E-5</c:v>
                 </c:pt>
                 <c:pt idx="29" formatCode="0.00E+00">
-                  <c:v>6.618761208503814E-5</c:v>
+                  <c:v>6.4951313743930733E-5</c:v>
                 </c:pt>
                 <c:pt idx="30" formatCode="0.00E+00">
-                  <c:v>6.7514921819445285E-5</c:v>
+                  <c:v>6.6253831062187442E-5</c:v>
                 </c:pt>
                 <c:pt idx="31" formatCode="0.00E+00">
-                  <c:v>6.8842231553851996E-5</c:v>
+                  <c:v>6.7556348380444584E-5</c:v>
                 </c:pt>
                 <c:pt idx="32" formatCode="0.00E+00">
-                  <c:v>7.0169541288259141E-5</c:v>
+                  <c:v>6.8858865698701293E-5</c:v>
                 </c:pt>
                 <c:pt idx="33" formatCode="0.00E+00">
-                  <c:v>7.1496851022665852E-5</c:v>
+                  <c:v>7.0161383016958435E-5</c:v>
                 </c:pt>
                 <c:pt idx="34" formatCode="0.00E+00">
-                  <c:v>7.2824160757072997E-5</c:v>
+                  <c:v>7.1463900335215144E-5</c:v>
                 </c:pt>
                 <c:pt idx="35" formatCode="0.00E+00">
-                  <c:v>7.4151470491480142E-5</c:v>
+                  <c:v>7.2766417653472287E-5</c:v>
                 </c:pt>
                 <c:pt idx="36" formatCode="0.00E+00">
-                  <c:v>7.5478780225886853E-5</c:v>
+                  <c:v>7.4068934971728995E-5</c:v>
                 </c:pt>
                 <c:pt idx="37" formatCode="0.00E+00">
-                  <c:v>7.6806089960293998E-5</c:v>
+                  <c:v>7.5371452289986138E-5</c:v>
                 </c:pt>
                 <c:pt idx="38" formatCode="0.00E+00">
-                  <c:v>7.8133399694700709E-5</c:v>
+                  <c:v>7.6673969608242847E-5</c:v>
                 </c:pt>
                 <c:pt idx="39" formatCode="0.00E+00">
-                  <c:v>7.977578850124848E-5</c:v>
+                  <c:v>7.8285680732168971E-5</c:v>
                 </c:pt>
                 <c:pt idx="40" formatCode="0.00E+00">
-                  <c:v>8.0968064347595233E-5</c:v>
+                  <c:v>7.9455686419425183E-5</c:v>
                 </c:pt>
                 <c:pt idx="41" formatCode="0.00E+00">
-                  <c:v>8.132511630401103E-5</c:v>
+                  <c:v>7.9806069110588361E-5</c:v>
                 </c:pt>
                 <c:pt idx="42" formatCode="0.00E+00">
-                  <c:v>8.4161072514692597E-5</c:v>
+                  <c:v>8.2589053354941577E-5</c:v>
                 </c:pt>
                 <c:pt idx="43" formatCode="0.00E+00">
-                  <c:v>8.498353764742068E-5</c:v>
+                  <c:v>8.3396155910788876E-5</c:v>
                 </c:pt>
                 <c:pt idx="44" formatCode="0.00E+00">
-                  <c:v>8.5775402347925225E-5</c:v>
+                  <c:v>8.4173229610609506E-5</c:v>
                 </c:pt>
                 <c:pt idx="45" formatCode="0.00E+00">
-                  <c:v>8.6479330619128737E-5</c:v>
+                  <c:v>8.4864009419033756E-5</c:v>
                 </c:pt>
                 <c:pt idx="46" formatCode="0.00E+00">
-                  <c:v>8.7180851987329484E-5</c:v>
+                  <c:v>8.5552427282266762E-5</c:v>
                 </c:pt>
                 <c:pt idx="47" formatCode="0.00E+00">
-                  <c:v>8.7676327828293231E-5</c:v>
+                  <c:v>8.6038648280202556E-5</c:v>
                 </c:pt>
                 <c:pt idx="48" formatCode="0.00E+00">
-                  <c:v>8.808308415773043E-5</c:v>
+                  <c:v>8.6437806931471918E-5</c:v>
                 </c:pt>
                 <c:pt idx="49" formatCode="0.00E+00">
-                  <c:v>8.8443349127241298E-5</c:v>
+                  <c:v>8.6791342620833007E-5</c:v>
                 </c:pt>
                 <c:pt idx="50" formatCode="0.00E+00">
-                  <c:v>8.877490666338608E-5</c:v>
+                  <c:v>8.7116707094273078E-5</c:v>
                 </c:pt>
                 <c:pt idx="51" formatCode="0.00E+00">
-                  <c:v>8.9036788024627383E-5</c:v>
+                  <c:v>8.7373696852958087E-5</c:v>
                 </c:pt>
                 <c:pt idx="52" formatCode="0.00E+00">
-                  <c:v>8.9408940248032558E-5</c:v>
+                  <c:v>8.7738897757801631E-5</c:v>
                 </c:pt>
                 <c:pt idx="53" formatCode="0.00E+00">
-                  <c:v>8.9726171714716883E-5</c:v>
+                  <c:v>8.8050203754089717E-5</c:v>
                 </c:pt>
                 <c:pt idx="54" formatCode="0.00E+00">
-                  <c:v>8.9993423792437643E-5</c:v>
+                  <c:v>8.8312463911269213E-5</c:v>
                 </c:pt>
                 <c:pt idx="55" formatCode="0.00E+00">
-                  <c:v>9.0174807564025167E-5</c:v>
+                  <c:v>8.8490459670374438E-5</c:v>
                 </c:pt>
                 <c:pt idx="56" formatCode="0.00E+00">
-                  <c:v>9.038234516069701E-5</c:v>
+                  <c:v>8.8694120735193857E-5</c:v>
                 </c:pt>
                 <c:pt idx="57" formatCode="0.00E+00">
-                  <c:v>9.0953441555838329E-5</c:v>
+                  <c:v>8.9254549793900385E-5</c:v>
                 </c:pt>
                 <c:pt idx="58" formatCode="0.00E+00">
-                  <c:v>9.1765196895077241E-5</c:v>
+                  <c:v>9.005114260124438E-5</c:v>
                 </c:pt>
                 <c:pt idx="59" formatCode="0.00E+00">
-                  <c:v>9.2611810298042204E-5</c:v>
+                  <c:v>9.0881942369109463E-5</c:v>
                 </c:pt>
                 <c:pt idx="60" formatCode="0.00E+00">
-                  <c:v>9.3647517531163859E-5</c:v>
+                  <c:v>9.1898303940802261E-5</c:v>
                 </c:pt>
                 <c:pt idx="61" formatCode="0.00E+00">
-                  <c:v>9.5050006294872494E-5</c:v>
+                  <c:v>9.3274596042063404E-5</c:v>
                 </c:pt>
                 <c:pt idx="62" formatCode="0.00E+00">
-                  <c:v>9.645662760019035E-5</c:v>
+                  <c:v>9.4654943494441841E-5</c:v>
                 </c:pt>
                 <c:pt idx="63" formatCode="0.00E+00">
-                  <c:v>9.7387214206997634E-5</c:v>
+                  <c:v>9.5568147956131454E-5</c:v>
                 </c:pt>
                 <c:pt idx="64" formatCode="0.00E+00">
-                  <c:v>9.8272881152577143E-5</c:v>
+                  <c:v>9.643727179732782E-5</c:v>
                 </c:pt>
                 <c:pt idx="65" formatCode="0.00E+00">
-                  <c:v>9.9315311676914197E-5</c:v>
+                  <c:v>9.7460231077917589E-5</c:v>
                 </c:pt>
                 <c:pt idx="66" formatCode="0.00E+00">
-                  <c:v>1.0022913979744075E-4</c:v>
+                  <c:v>9.8356990080011308E-5</c:v>
                 </c:pt>
                 <c:pt idx="67" formatCode="0.00E+00">
-                  <c:v>1.0111291012785455E-4</c:v>
+                  <c:v>9.9224252732341657E-5</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -16437,88 +16437,88 @@
         <v>1.0877081887028839E-4</v>
       </c>
       <c r="F9" s="4">
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="G9" s="4">
-        <v>8.132511630401103E-5</v>
+        <v>7.9806069110588361E-5</v>
       </c>
       <c r="H9" s="4">
-        <v>8.4161072514692597E-5</v>
+        <v>8.2589053354941577E-5</v>
       </c>
       <c r="I9" s="4">
-        <v>8.498353764742068E-5</v>
+        <v>8.3396155910788876E-5</v>
       </c>
       <c r="J9" s="4">
-        <v>8.5775402347925225E-5</v>
+        <v>8.4173229610609506E-5</v>
       </c>
       <c r="K9" s="4">
-        <v>8.6479330619128737E-5</v>
+        <v>8.4864009419033756E-5</v>
       </c>
       <c r="L9" s="4">
-        <v>8.7180851987329484E-5</v>
+        <v>8.5552427282266762E-5</v>
       </c>
       <c r="M9" s="4">
-        <v>8.7676327828293231E-5</v>
+        <v>8.6038648280202556E-5</v>
       </c>
       <c r="N9" s="4">
-        <v>8.808308415773043E-5</v>
+        <v>8.6437806931471918E-5</v>
       </c>
       <c r="O9" s="4">
-        <v>8.8443349127241298E-5</v>
+        <v>8.6791342620833007E-5</v>
       </c>
       <c r="P9" s="4">
-        <v>8.877490666338608E-5</v>
+        <v>8.7116707094273078E-5</v>
       </c>
       <c r="Q9" s="4">
-        <v>8.9036788024627383E-5</v>
+        <v>8.7373696852958087E-5</v>
       </c>
       <c r="R9" s="4">
-        <v>8.9408940248032558E-5</v>
+        <v>8.7738897757801631E-5</v>
       </c>
       <c r="S9" s="4">
-        <v>8.9726171714716883E-5</v>
+        <v>8.8050203754089717E-5</v>
       </c>
       <c r="T9" s="4">
-        <v>8.9993423792437643E-5</v>
+        <v>8.8312463911269213E-5</v>
       </c>
       <c r="U9" s="4">
-        <v>9.0174807564025167E-5</v>
+        <v>8.8490459670374438E-5</v>
       </c>
       <c r="V9" s="4">
-        <v>9.038234516069701E-5</v>
+        <v>8.8694120735193857E-5</v>
       </c>
       <c r="W9" s="4">
-        <v>9.0953441555838329E-5</v>
+        <v>8.9254549793900385E-5</v>
       </c>
       <c r="X9" s="4">
-        <v>9.1765196895077241E-5</v>
+        <v>9.005114260124438E-5</v>
       </c>
       <c r="Y9" s="4">
-        <v>9.2611810298042204E-5</v>
+        <v>9.0881942369109463E-5</v>
       </c>
       <c r="Z9" s="4">
-        <v>9.3647517531163859E-5</v>
+        <v>9.1898303940802261E-5</v>
       </c>
       <c r="AA9" s="4">
-        <v>9.5050006294872494E-5</v>
+        <v>9.3274596042063404E-5</v>
       </c>
       <c r="AB9" s="4">
-        <v>9.645662760019035E-5</v>
+        <v>9.4654943494441841E-5</v>
       </c>
       <c r="AC9" s="4">
-        <v>9.7387214206997634E-5</v>
+        <v>9.5568147956131454E-5</v>
       </c>
       <c r="AD9" s="4">
-        <v>9.8272881152577143E-5</v>
+        <v>9.643727179732782E-5</v>
       </c>
       <c r="AE9" s="4">
-        <v>9.9315311676914197E-5</v>
+        <v>9.7460231077917589E-5</v>
       </c>
       <c r="AF9" s="4">
-        <v>1.0022913979744075E-4</v>
+        <v>9.8356990080011308E-5</v>
       </c>
       <c r="AG9" s="4">
-        <v>1.0111291012785455E-4</v>
+        <v>9.9224252732341657E-5</v>
       </c>
       <c r="AH9" s="4"/>
       <c r="AI9" s="4"/>
@@ -18660,22 +18660,22 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="C10" s="4">
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="D10" s="4">
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="E10" s="4">
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="F10">
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="G10" s="4">
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="H10" s="4">
         <v>8.379890176963306E-5</v>
@@ -19656,179 +19656,179 @@
       <c r="Z3" s="23"/>
       <c r="AA3" s="4" cm="1">
         <f t="array" ref="AA3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AA1)</f>
-        <v>5.9551063413003282E-5</v>
+        <v>5.8438727152645888E-5</v>
       </c>
       <c r="AB3" s="4" cm="1">
         <f t="array" ref="AB3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AB1)</f>
-        <v>6.0878373147410427E-5</v>
+        <v>5.9741244470903031E-5</v>
       </c>
       <c r="AC3" s="4" cm="1">
         <f t="array" ref="AC3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AC1)</f>
-        <v>6.2205682881817138E-5</v>
+        <v>6.1043761789159739E-5</v>
       </c>
       <c r="AD3" s="4" cm="1">
         <f t="array" ref="AD3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AD1)</f>
-        <v>6.3532992616224283E-5</v>
+        <v>6.2346279107416882E-5</v>
       </c>
       <c r="AE3" s="4" cm="1">
         <f t="array" ref="AE3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AE1)</f>
-        <v>6.4860302350631428E-5</v>
+        <v>6.3648796425673591E-5</v>
       </c>
       <c r="AF3" s="4" cm="1">
         <f t="array" ref="AF3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AF1)</f>
-        <v>6.618761208503814E-5</v>
+        <v>6.4951313743930733E-5</v>
       </c>
       <c r="AG3" s="4" cm="1">
         <f t="array" ref="AG3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AG1)</f>
-        <v>6.7514921819445285E-5</v>
+        <v>6.6253831062187442E-5</v>
       </c>
       <c r="AH3" s="4" cm="1">
         <f t="array" ref="AH3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AH1)</f>
-        <v>6.8842231553851996E-5</v>
+        <v>6.7556348380444584E-5</v>
       </c>
       <c r="AI3" s="4" cm="1">
         <f t="array" ref="AI3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AI1)</f>
-        <v>7.0169541288259141E-5</v>
+        <v>6.8858865698701293E-5</v>
       </c>
       <c r="AJ3" s="4" cm="1">
         <f t="array" ref="AJ3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AJ1)</f>
-        <v>7.1496851022665852E-5</v>
+        <v>7.0161383016958435E-5</v>
       </c>
       <c r="AK3" s="4" cm="1">
         <f t="array" ref="AK3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AK1)</f>
-        <v>7.2824160757072997E-5</v>
+        <v>7.1463900335215144E-5</v>
       </c>
       <c r="AL3" s="4" cm="1">
         <f t="array" ref="AL3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AL1)</f>
-        <v>7.4151470491480142E-5</v>
+        <v>7.2766417653472287E-5</v>
       </c>
       <c r="AM3" s="4" cm="1">
         <f t="array" ref="AM3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AM1)</f>
-        <v>7.5478780225886853E-5</v>
+        <v>7.4068934971728995E-5</v>
       </c>
       <c r="AN3" s="4" cm="1">
         <f t="array" ref="AN3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AN1)</f>
-        <v>7.6806089960293998E-5</v>
+        <v>7.5371452289986138E-5</v>
       </c>
       <c r="AO3" s="4" cm="1">
         <f t="array" ref="AO3">TREND($AQ$3:$AU$3,$AQ$1:$AU$1,AO1)</f>
-        <v>7.8133399694700709E-5</v>
+        <v>7.6673969608242847E-5</v>
       </c>
       <c r="AP3" s="4" cm="1">
         <f t="array" ref="AP3">TREND($AR$3:$AV$3,$AR$1:$AV$1,AP1)</f>
-        <v>7.977578850124848E-5</v>
+        <v>7.8285680732168971E-5</v>
       </c>
       <c r="AQ3" s="4" cm="1">
         <f t="array" ref="AQ3">TREND($AR$3:$AV$3,$AR$1:$AV$1,AQ1)</f>
-        <v>8.0968064347595233E-5</v>
+        <v>7.9455686419425183E-5</v>
       </c>
       <c r="AR3" s="20">
         <f>BNVFE!G9</f>
-        <v>8.132511630401103E-5</v>
+        <v>7.9806069110588361E-5</v>
       </c>
       <c r="AS3" s="26">
         <f>BNVFE!H9</f>
-        <v>8.4161072514692597E-5</v>
+        <v>8.2589053354941577E-5</v>
       </c>
       <c r="AT3" s="26">
         <f>BNVFE!I9</f>
-        <v>8.498353764742068E-5</v>
+        <v>8.3396155910788876E-5</v>
       </c>
       <c r="AU3" s="26">
         <f>BNVFE!J9</f>
-        <v>8.5775402347925225E-5</v>
+        <v>8.4173229610609506E-5</v>
       </c>
       <c r="AV3" s="26">
         <f>BNVFE!K9</f>
-        <v>8.6479330619128737E-5</v>
+        <v>8.4864009419033756E-5</v>
       </c>
       <c r="AW3" s="26">
         <f>BNVFE!L9</f>
-        <v>8.7180851987329484E-5</v>
+        <v>8.5552427282266762E-5</v>
       </c>
       <c r="AX3" s="26">
         <f>BNVFE!M9</f>
-        <v>8.7676327828293231E-5</v>
+        <v>8.6038648280202556E-5</v>
       </c>
       <c r="AY3" s="26">
         <f>BNVFE!N9</f>
-        <v>8.808308415773043E-5</v>
+        <v>8.6437806931471918E-5</v>
       </c>
       <c r="AZ3" s="26">
         <f>BNVFE!O9</f>
-        <v>8.8443349127241298E-5</v>
+        <v>8.6791342620833007E-5</v>
       </c>
       <c r="BA3" s="26">
         <f>BNVFE!P9</f>
-        <v>8.877490666338608E-5</v>
+        <v>8.7116707094273078E-5</v>
       </c>
       <c r="BB3" s="26">
         <f>BNVFE!Q9</f>
-        <v>8.9036788024627383E-5</v>
+        <v>8.7373696852958087E-5</v>
       </c>
       <c r="BC3" s="26">
         <f>BNVFE!R9</f>
-        <v>8.9408940248032558E-5</v>
+        <v>8.7738897757801631E-5</v>
       </c>
       <c r="BD3" s="26">
         <f>BNVFE!S9</f>
-        <v>8.9726171714716883E-5</v>
+        <v>8.8050203754089717E-5</v>
       </c>
       <c r="BE3" s="26">
         <f>BNVFE!T9</f>
-        <v>8.9993423792437643E-5</v>
+        <v>8.8312463911269213E-5</v>
       </c>
       <c r="BF3" s="26">
         <f>BNVFE!U9</f>
-        <v>9.0174807564025167E-5</v>
+        <v>8.8490459670374438E-5</v>
       </c>
       <c r="BG3" s="26">
         <f>BNVFE!V9</f>
-        <v>9.038234516069701E-5</v>
+        <v>8.8694120735193857E-5</v>
       </c>
       <c r="BH3" s="26">
         <f>BNVFE!W9</f>
-        <v>9.0953441555838329E-5</v>
+        <v>8.9254549793900385E-5</v>
       </c>
       <c r="BI3" s="26">
         <f>BNVFE!X9</f>
-        <v>9.1765196895077241E-5</v>
+        <v>9.005114260124438E-5</v>
       </c>
       <c r="BJ3" s="26">
         <f>BNVFE!Y9</f>
-        <v>9.2611810298042204E-5</v>
+        <v>9.0881942369109463E-5</v>
       </c>
       <c r="BK3" s="26">
         <f>BNVFE!Z9</f>
-        <v>9.3647517531163859E-5</v>
+        <v>9.1898303940802261E-5</v>
       </c>
       <c r="BL3" s="26">
         <f>BNVFE!AA9</f>
-        <v>9.5050006294872494E-5</v>
+        <v>9.3274596042063404E-5</v>
       </c>
       <c r="BM3" s="26">
         <f>BNVFE!AB9</f>
-        <v>9.645662760019035E-5</v>
+        <v>9.4654943494441841E-5</v>
       </c>
       <c r="BN3" s="26">
         <f>BNVFE!AC9</f>
-        <v>9.7387214206997634E-5</v>
+        <v>9.5568147956131454E-5</v>
       </c>
       <c r="BO3" s="26">
         <f>BNVFE!AD9</f>
-        <v>9.8272881152577143E-5</v>
+        <v>9.643727179732782E-5</v>
       </c>
       <c r="BP3" s="26">
         <f>BNVFE!AE9</f>
-        <v>9.9315311676914197E-5</v>
+        <v>9.7460231077917589E-5</v>
       </c>
       <c r="BQ3" s="26">
         <f>BNVFE!AF9</f>
-        <v>1.0022913979744075E-4</v>
+        <v>9.8356990080011308E-5</v>
       </c>
       <c r="BR3" s="26">
         <f>BNVFE!AG9</f>
-        <v>1.0111291012785455E-4</v>
+        <v>9.9224252732341657E-5</v>
       </c>
       <c r="BS3" s="26"/>
       <c r="BT3" s="4"/>
@@ -23788,123 +23788,123 @@
       </c>
       <c r="B2" s="4">
         <f t="array" ref="B2:B8">TRANSPOSE(SYFAFE!B10:H10)</f>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="C2" s="4">
         <f>B2</f>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="D2" s="4">
         <f t="shared" ref="D2:AE8" si="0">C2</f>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="E2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="F2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="G2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="K2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="L2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="M2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="N2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="O2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="P2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="Q2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="R2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="S2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="T2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="U2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="V2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="W2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="X2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="Y2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="Z2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="AA2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="AB2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="AC2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="AD2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="AE2" s="4">
         <f t="shared" si="0"/>
-        <v>3.0636736837912965E-4</v>
+        <v>3.0156650473713915E-4</v>
       </c>
       <c r="AG2" s="4"/>
       <c r="AH2" s="4"/>
@@ -23914,123 +23914,123 @@
         <v>3</v>
       </c>
       <c r="B3" s="4">
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="C3" s="4">
         <f t="shared" ref="C3:C8" si="1">B3</f>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="D3" s="4">
         <f t="shared" ref="D3:Q3" si="2">C3</f>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="F3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="G3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="H3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="I3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="J3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="K3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="L3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="M3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="N3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="O3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="P3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="Q3" s="4">
         <f t="shared" si="2"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="R3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="S3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="T3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="U3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="V3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="W3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="X3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="Y3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="Z3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="AA3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="AB3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="AC3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="AD3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="AE3" s="4">
         <f t="shared" si="0"/>
-        <v>7.273085411263018E-5</v>
+        <v>7.0213473556835903E-5</v>
       </c>
       <c r="AG3" s="4"/>
       <c r="AH3" s="4"/>
@@ -24040,123 +24040,123 @@
         <v>4</v>
       </c>
       <c r="B4" s="4">
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" si="1"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="D4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="F4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="G4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="H4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="I4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="J4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="K4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="L4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="N4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="O4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="P4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="Q4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="R4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="S4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="T4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="U4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="V4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="W4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="X4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="Y4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="Z4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="AA4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="AB4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="AC4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="AD4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="AE4" s="4">
         <f t="shared" si="0"/>
-        <v>9.5098581742816967E-5</v>
+        <v>9.3322264163941547E-5</v>
       </c>
       <c r="AG4" s="4"/>
       <c r="AH4" s="4"/>
@@ -24166,123 +24166,123 @@
         <v>5</v>
       </c>
       <c r="B5" s="4">
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="1"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="D5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="F5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="G5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="H5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="I5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="J5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="K5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="L5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="N5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="O5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="P5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="Q5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="R5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="S5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="T5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="U5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="V5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="W5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="X5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="Y5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="Z5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="AA5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="AB5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="AC5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="AD5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="AE5" s="4">
         <f t="shared" si="0"/>
-        <v>9.3478062847081558E-5</v>
+        <v>8.9590243650741159E-5</v>
       </c>
       <c r="AG5" s="4"/>
       <c r="AH5" s="4"/>
@@ -24292,123 +24292,123 @@
         <v>6</v>
       </c>
       <c r="B6" s="4">
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="1"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="D6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="F6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="G6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="H6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="I6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="J6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="K6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="L6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="M6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="N6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="O6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="P6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="Q6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="R6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="S6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="T6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="U6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="V6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="W6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="X6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="Y6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="Z6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="AA6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="AB6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="AC6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="AD6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="AE6" s="4">
         <f t="shared" si="0"/>
-        <v>3.8357149864294821E-5</v>
+        <v>1.5342859945717928E-4</v>
       </c>
       <c r="AG6" s="4"/>
       <c r="AH6" s="4"/>
@@ -24418,123 +24418,123 @@
         <v>84</v>
       </c>
       <c r="B7" s="4">
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="1"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="D7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="F7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="G7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="H7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="I7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="J7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="K7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="L7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="M7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="N7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="O7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="P7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="Q7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="R7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="S7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="T7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="U7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="V7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="W7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="X7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="Y7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="Z7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="AA7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="AB7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="AC7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="AD7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="AE7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4090027704705712E-3</v>
+        <v>1.1549320628198341E-4</v>
       </c>
       <c r="AG7" s="4"/>
       <c r="AH7" s="4"/>

</xml_diff>

<commit_message>
Rebase transportation files relying on 2024 to use AEO 2026 and extrpolating 2025 back one year; this avoids large jumps due to methodology shifts between AEO 2025 and AEO 2026
</commit_message>
<xml_diff>
--- a/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
+++ b/InputData/trans/BHNVFEAL/BAU Historical New Veh Fuel Economy After Lifetime.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\trans\BHNVFEAL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\BHNVFEAL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46122336-199E-4D3F-9ABC-740C7AD03B73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B49189A5-499E-4812-B686-83989CBCADAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="615" yWindow="45" windowWidth="20370" windowHeight="17025" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1520" yWindow="1520" windowWidth="19200" windowHeight="10050" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -53,6 +53,7 @@
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
         <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -82,7 +83,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="291" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="298" uniqueCount="106">
   <si>
     <t>Sources:</t>
   </si>
@@ -379,6 +380,27 @@
   </si>
   <si>
     <t>energy consumption that more closely matches EIA's AEO trajectory: freight LDVs, passenger HDVs, freight HDVs, passenger ships, passenger motorbikes.</t>
+  </si>
+  <si>
+    <t>Motorbike fuel-economy refresh (2026-09-03, pending staff review):</t>
+  </si>
+  <si>
+    <t>The internal 'SYFAFE' tab's passenger motorbike row was refreshed from the SYFAFE workbook, where</t>
+  </si>
+  <si>
+    <t>motorbike fuel economy was re-derived after replacing the old x5 activity calibration multiplier with</t>
+  </si>
+  <si>
+    <t>FHWA VM-1 2024 data (gasoline 0.00182 -&gt; 0.00050 passenger-miles/BTU; see the SYFAFE and BAADTbVT</t>
+  </si>
+  <si>
+    <t>About tabs and memo-aeo-vmt-seam-2026-08-31.md at the repo root). The BHNVFEAL motorbike outputs are</t>
+  </si>
+  <si>
+    <t>the SYFAFE motorbike row held flat across historical years, so they update with it. Note the motorbike</t>
+  </si>
+  <si>
+    <t>outputs read the SYFAFE tab, not the BNVFE tab.</t>
   </si>
 </sst>
 </file>
@@ -7784,11 +7806,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B48"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:B56"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="13.42578125" customWidth="1"/>
-    <col min="2" max="2" width="107.42578125" customWidth="1"/>
+    <col min="1" max="1" width="13.453125" customWidth="1"/>
+    <col min="2" max="2" width="107.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -7994,6 +8016,41 @@
     <row r="48" spans="1:1">
       <c r="A48" t="s">
         <v>98</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1">
+      <c r="A50" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1">
+      <c r="A51" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1">
+      <c r="A52" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1">
+      <c r="A53" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1">
+      <c r="A54" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1">
+      <c r="A55" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1">
+      <c r="A56" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -8011,12 +8068,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -9005,13 +9062,13 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
-    <col min="2" max="2" width="21.28515625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="2" max="2" width="21.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -9878,12 +9935,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -10750,14 +10807,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AF13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
-    <col min="2" max="2" width="10.42578125" customWidth="1"/>
-    <col min="3" max="3" width="10.7109375" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
+    <col min="2" max="2" width="10.453125" customWidth="1"/>
+    <col min="3" max="3" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="30">
+    <row r="1" spans="1:32">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -11651,12 +11708,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -12523,12 +12580,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -13509,12 +13566,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -14381,12 +14438,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -14487,123 +14544,123 @@
       </c>
       <c r="B2" s="4">
         <f t="array" ref="B2:B8">TRANSPOSE(SYFAFE!B7:H7)</f>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="C2" s="4">
         <f>B2</f>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="D2" s="4">
         <f t="shared" ref="D2:AE8" si="0">C2</f>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="E2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="F2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="G2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="H2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="I2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="J2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="K2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="L2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="M2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="N2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="O2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="P2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="Q2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="R2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="S2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="T2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="U2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="V2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="W2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="X2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="Y2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="Z2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="AA2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="AB2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="AC2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="AD2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="AE2" s="4">
         <f t="shared" si="0"/>
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="AG2" s="4"/>
       <c r="AH2" s="4"/>
@@ -14613,123 +14670,123 @@
         <v>3</v>
       </c>
       <c r="B3" s="4">
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="C3" s="4">
         <f t="shared" ref="C3:C8" si="1">B3</f>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="D3" s="4">
         <f t="shared" ref="D3:Q3" si="2">C3</f>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="E3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="F3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="G3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="H3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="I3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="J3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="K3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="L3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="M3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="N3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="O3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="P3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Q3" s="4">
         <f t="shared" si="2"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="R3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="S3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="T3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="U3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="V3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="W3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="X3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Y3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Z3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AA3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AB3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AC3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AD3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AE3" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AG3" s="4"/>
       <c r="AH3" s="4"/>
@@ -14739,123 +14796,123 @@
         <v>4</v>
       </c>
       <c r="B4" s="4">
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" si="1"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="D4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="F4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="G4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="H4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="I4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="J4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="K4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="L4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="M4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="N4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="O4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="P4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Q4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="R4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="S4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="T4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="U4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="V4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="W4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="X4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Y4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Z4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AA4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AB4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AC4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AD4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AE4" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AG4" s="4"/>
       <c r="AH4" s="4"/>
@@ -14865,123 +14922,123 @@
         <v>5</v>
       </c>
       <c r="B5" s="4">
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="1"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="D5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="F5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="G5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="H5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="I5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="J5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="K5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="L5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="M5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="N5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="O5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="P5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Q5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="R5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="S5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="T5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="U5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="V5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="W5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="X5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Y5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="Z5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AA5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AB5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AC5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AD5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AE5" s="4">
         <f t="shared" si="0"/>
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="AG5" s="4"/>
       <c r="AH5" s="4"/>
@@ -14991,123 +15048,123 @@
         <v>6</v>
       </c>
       <c r="B6" s="4">
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="1"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="D6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="F6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="G6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="H6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="I6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="J6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="K6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="L6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="M6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="N6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="O6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="P6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="Q6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="R6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="S6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="T6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="U6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="V6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="W6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="X6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="Y6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="Z6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="AA6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="AB6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="AC6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="AD6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="AE6" s="4">
         <f t="shared" si="0"/>
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="AG6" s="4"/>
       <c r="AH6" s="4"/>
@@ -15117,123 +15174,123 @@
         <v>84</v>
       </c>
       <c r="B7" s="4">
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="1"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="D7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="F7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="G7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="H7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="I7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="J7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="K7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="L7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="M7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="N7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="O7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="P7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="Q7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="R7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="S7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="T7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="U7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="V7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="W7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="X7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="Y7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="Z7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="AA7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="AB7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="AC7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="AD7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="AE7" s="4">
         <f t="shared" si="0"/>
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="AG7" s="4"/>
       <c r="AH7" s="4"/>
@@ -15243,123 +15300,123 @@
         <v>85</v>
       </c>
       <c r="B8" s="4">
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" si="1"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="D8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="F8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="G8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="H8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="I8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="J8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="K8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="L8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="M8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="N8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="O8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="P8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="Q8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="R8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="S8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="T8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="U8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="V8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="W8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="X8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="Y8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="Z8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="AA8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="AB8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="AC8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="AD8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="AE8" s="4">
         <f t="shared" si="0"/>
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
       <c r="AG8" s="4"/>
       <c r="AH8" s="4"/>
@@ -15375,12 +15432,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" ht="30">
+    <row r="1" spans="1:31">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -16148,11 +16205,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AK30"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" customWidth="1"/>
-    <col min="2" max="2" width="16.42578125" customWidth="1"/>
-    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="1" max="1" width="18.453125" customWidth="1"/>
+    <col min="2" max="2" width="16.453125" customWidth="1"/>
+    <col min="3" max="3" width="30.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37">
@@ -18445,7 +18502,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:8">
       <c r="A1" t="s">
@@ -18608,25 +18665,25 @@
         <v>18</v>
       </c>
       <c r="B7">
-        <v>5.8028780082485321E-3</v>
+        <v>1.583802E-3</v>
       </c>
       <c r="C7">
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="D7">
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="E7">
-        <v>1.8223914406069774E-3</v>
+        <v>4.9739300000000005E-4</v>
       </c>
       <c r="F7">
-        <v>4.0116590528098328E-3</v>
+        <v>1.0949180000000001E-3</v>
       </c>
       <c r="G7">
-        <v>1.4123533664704075E-3</v>
+        <v>3.8547899999999999E-4</v>
       </c>
       <c r="H7">
-        <v>5.467174321820931E-3</v>
+        <v>1.492178E-3</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -18819,9 +18876,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="50.42578125" customWidth="1"/>
+    <col min="1" max="1" width="50.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -18923,11 +18980,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:AL31"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="42.140625" customWidth="1"/>
-    <col min="2" max="2" width="26.42578125" customWidth="1"/>
-    <col min="3" max="3" width="42.85546875" customWidth="1"/>
+    <col min="1" max="1" width="42.1796875" customWidth="1"/>
+    <col min="2" max="2" width="26.453125" customWidth="1"/>
+    <col min="3" max="3" width="42.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:38">
@@ -19097,7 +19154,7 @@
         <v>5.76</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="30">
+    <row r="20" spans="1:4" ht="29">
       <c r="A20" s="9" t="s">
         <v>68</v>
       </c>
@@ -19115,7 +19172,7 @@
         <v>6.7042622950819668</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="30">
+    <row r="22" spans="1:4" ht="29">
       <c r="A22" s="9" t="s">
         <v>70</v>
       </c>
@@ -19201,10 +19258,10 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:BT15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="15" max="15" width="11.42578125" customWidth="1"/>
+    <col min="15" max="15" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:72">
@@ -22648,12 +22705,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -23682,12 +23739,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>
@@ -24676,12 +24733,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AH8"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="31.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" ht="30">
+    <row r="1" spans="1:34">
       <c r="A1" s="14" t="s">
         <v>87</v>
       </c>

</xml_diff>